<commit_message>
last updated on main branch before validation begins
</commit_message>
<xml_diff>
--- a/src/inputs/canonical_nodes.xlsx
+++ b/src/inputs/canonical_nodes.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ben/Documents/bruegel/data_new/WORKING/INDUSTRY/tuone_v5/src/inputs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ben/Documents/bruegel/data_new/WORKING/INDUSTRY/tuone_v6/src/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEB00877-9B1B-874B-97C2-FFC20D42DC55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B54FB752-40EC-0644-9FD6-1585903B04FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4500" yWindow="500" windowWidth="29400" windowHeight="16940" xr2:uid="{EBC50A8D-91C7-594D-A950-AF99F2B3F4AF}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="16940" xr2:uid="{EBC50A8D-91C7-594D-A950-AF99F2B3F4AF}"/>
   </bookViews>
   <sheets>
     <sheet name="merge" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="98">
   <si>
     <t>Pylon LifeEU</t>
   </si>
@@ -322,6 +322,15 @@
   </si>
   <si>
     <t>Ciel &amp; Terre</t>
+  </si>
+  <si>
+    <t>Engie</t>
+  </si>
+  <si>
+    <t>Vilvoorde</t>
+  </si>
+  <si>
+    <t>Vilvorde</t>
   </si>
 </sst>
 </file>
@@ -709,7 +718,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DF9B3CA-7DC7-BB45-882F-C1DDB5BD93A3}">
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.5" bestFit="1" customWidth="1"/>
@@ -1474,6 +1483,34 @@
       </c>
       <c r="D54" t="s">
         <v>94</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>63</v>
+      </c>
+      <c r="B55" t="s">
+        <v>64</v>
+      </c>
+      <c r="C55" t="s">
+        <v>65</v>
+      </c>
+      <c r="D55" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>96</v>
+      </c>
+      <c r="B56" t="s">
+        <v>95</v>
+      </c>
+      <c r="C56" t="s">
+        <v>97</v>
+      </c>
+      <c r="D56" t="s">
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
validating battery cell projects
</commit_message>
<xml_diff>
--- a/src/inputs/canonical_nodes.xlsx
+++ b/src/inputs/canonical_nodes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ben/Documents/bruegel/data_new/WORKING/INDUSTRY/tuone_v6/src/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B54FB752-40EC-0644-9FD6-1585903B04FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3405E14-29FF-1F4A-8EDF-2026411D2634}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="16940" xr2:uid="{EBC50A8D-91C7-594D-A950-AF99F2B3F4AF}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="125">
   <si>
     <t>Pylon LifeEU</t>
   </si>
@@ -331,6 +331,87 @@
   </si>
   <si>
     <t>Vilvorde</t>
+  </si>
+  <si>
+    <t>Coventry</t>
+  </si>
+  <si>
+    <t>Eve Energy</t>
+  </si>
+  <si>
+    <t>West Midlands</t>
+  </si>
+  <si>
+    <t>Erfurt</t>
+  </si>
+  <si>
+    <t>Arnstadt</t>
+  </si>
+  <si>
+    <t>Thuringia</t>
+  </si>
+  <si>
+    <t>Thüringen</t>
+  </si>
+  <si>
+    <t>Berlin</t>
+  </si>
+  <si>
+    <t>Giga Berlin</t>
+  </si>
+  <si>
+    <t>Grünheide</t>
+  </si>
+  <si>
+    <t>Berlin-Brandenburg</t>
+  </si>
+  <si>
+    <t>Brandenburg</t>
+  </si>
+  <si>
+    <t>Giga-Berlin</t>
+  </si>
+  <si>
+    <t>GigaBerlin</t>
+  </si>
+  <si>
+    <t>Gruenheide</t>
+  </si>
+  <si>
+    <t>Blyth</t>
+  </si>
+  <si>
+    <t>Britishvolt</t>
+  </si>
+  <si>
+    <t>Cambois</t>
+  </si>
+  <si>
+    <t>Northumberland</t>
+  </si>
+  <si>
+    <t>Bridgewater</t>
+  </si>
+  <si>
+    <t>Bridgwater</t>
+  </si>
+  <si>
+    <t>Tata Group</t>
+  </si>
+  <si>
+    <t>Somerset</t>
+  </si>
+  <si>
+    <t>Douvrin</t>
+  </si>
+  <si>
+    <t>Agder</t>
+  </si>
+  <si>
+    <t>Morrow Batteries</t>
+  </si>
+  <si>
+    <t>Arendal</t>
   </si>
 </sst>
 </file>
@@ -718,7 +799,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DF9B3CA-7DC7-BB45-882F-C1DDB5BD93A3}">
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E73"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.5" bestFit="1" customWidth="1"/>
@@ -745,461 +826,461 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>27</v>
+        <v>93</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
+        <v>86</v>
       </c>
       <c r="C2" t="s">
-        <v>29</v>
+        <v>93</v>
       </c>
       <c r="D2" t="s">
-        <v>28</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>76</v>
+        <v>27</v>
       </c>
       <c r="B3" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>76</v>
+        <v>29</v>
       </c>
       <c r="D3" t="s">
-        <v>77</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>30</v>
+        <v>76</v>
       </c>
       <c r="B4" t="s">
-        <v>31</v>
+        <v>75</v>
       </c>
       <c r="C4" t="s">
-        <v>32</v>
+        <v>76</v>
       </c>
       <c r="D4" t="s">
-        <v>31</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>113</v>
       </c>
       <c r="B5" t="s">
-        <v>31</v>
+        <v>114</v>
       </c>
       <c r="C5" t="s">
-        <v>32</v>
+        <v>115</v>
       </c>
       <c r="D5" t="s">
-        <v>31</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>30</v>
+        <v>113</v>
       </c>
       <c r="B6" t="s">
-        <v>31</v>
+        <v>114</v>
       </c>
       <c r="C6" t="s">
-        <v>30</v>
+        <v>116</v>
       </c>
       <c r="D6" t="s">
-        <v>33</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>30</v>
+        <v>118</v>
       </c>
       <c r="B7" t="s">
-        <v>31</v>
+        <v>119</v>
       </c>
       <c r="C7" t="s">
-        <v>30</v>
+        <v>117</v>
       </c>
       <c r="D7" t="s">
-        <v>34</v>
+        <v>119</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>30</v>
+        <v>118</v>
       </c>
       <c r="B8" t="s">
-        <v>31</v>
+        <v>119</v>
       </c>
       <c r="C8" t="s">
-        <v>30</v>
+        <v>120</v>
       </c>
       <c r="D8" t="s">
-        <v>35</v>
+        <v>119</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="B9" t="s">
-        <v>66</v>
+        <v>86</v>
       </c>
       <c r="C9" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="D9" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="B10" t="s">
-        <v>71</v>
+        <v>31</v>
       </c>
       <c r="C10" t="s">
-        <v>70</v>
+        <v>32</v>
       </c>
       <c r="D10" t="s">
-        <v>72</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="B11" t="s">
-        <v>71</v>
+        <v>31</v>
       </c>
       <c r="C11" t="s">
-        <v>70</v>
+        <v>32</v>
       </c>
       <c r="D11" t="s">
-        <v>73</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="B12" t="s">
-        <v>71</v>
+        <v>31</v>
       </c>
       <c r="C12" t="s">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="D12" t="s">
-        <v>74</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="B13" t="s">
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="C13" t="s">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="D13" t="s">
-        <v>7</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>78</v>
+        <v>30</v>
       </c>
       <c r="B14" t="s">
-        <v>79</v>
+        <v>31</v>
       </c>
       <c r="C14" t="s">
-        <v>78</v>
+        <v>30</v>
       </c>
       <c r="D14" t="s">
-        <v>80</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>78</v>
+        <v>98</v>
       </c>
       <c r="B15" t="s">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="C15" t="s">
-        <v>78</v>
+        <v>100</v>
       </c>
       <c r="D15" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>62</v>
+        <v>101</v>
       </c>
       <c r="B16" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="C16" t="s">
-        <v>62</v>
+        <v>102</v>
       </c>
       <c r="D16" t="s">
-        <v>60</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>62</v>
+        <v>101</v>
       </c>
       <c r="B17" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="C17" t="s">
-        <v>62</v>
+        <v>103</v>
       </c>
       <c r="D17" t="s">
-        <v>52</v>
+        <v>84</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>21</v>
+        <v>101</v>
       </c>
       <c r="B18" t="s">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="C18" t="s">
-        <v>21</v>
+        <v>104</v>
       </c>
       <c r="D18" t="s">
-        <v>22</v>
+        <v>84</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>21</v>
+        <v>67</v>
       </c>
       <c r="B19" t="s">
-        <v>20</v>
+        <v>66</v>
       </c>
       <c r="C19" t="s">
-        <v>21</v>
+        <v>67</v>
       </c>
       <c r="D19" t="s">
-        <v>23</v>
+        <v>68</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>21</v>
+        <v>70</v>
       </c>
       <c r="B20" t="s">
-        <v>20</v>
+        <v>71</v>
       </c>
       <c r="C20" t="s">
-        <v>38</v>
+        <v>70</v>
       </c>
       <c r="D20" t="s">
-        <v>22</v>
+        <v>72</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>21</v>
+        <v>70</v>
       </c>
       <c r="B21" t="s">
-        <v>20</v>
+        <v>71</v>
       </c>
       <c r="C21" t="s">
-        <v>24</v>
+        <v>70</v>
       </c>
       <c r="D21" t="s">
-        <v>22</v>
+        <v>73</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>21</v>
+        <v>70</v>
       </c>
       <c r="B22" t="s">
-        <v>20</v>
+        <v>71</v>
       </c>
       <c r="C22" t="s">
-        <v>24</v>
+        <v>70</v>
       </c>
       <c r="D22" t="s">
-        <v>23</v>
+        <v>74</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>21</v>
+        <v>107</v>
       </c>
       <c r="B23" t="s">
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="C23" t="s">
-        <v>24</v>
+        <v>106</v>
       </c>
       <c r="D23" t="s">
-        <v>20</v>
+        <v>69</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>21</v>
+        <v>107</v>
       </c>
       <c r="B24" t="s">
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="C24" t="s">
-        <v>24</v>
+        <v>105</v>
       </c>
       <c r="D24" t="s">
-        <v>40</v>
+        <v>69</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>63</v>
+        <v>107</v>
       </c>
       <c r="B25" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="C25" t="s">
-        <v>65</v>
+        <v>108</v>
       </c>
       <c r="D25" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>57</v>
+        <v>107</v>
       </c>
       <c r="B26" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C26" t="s">
-        <v>57</v>
+        <v>109</v>
       </c>
       <c r="D26" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>59</v>
+        <v>107</v>
       </c>
       <c r="B27" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C27" t="s">
-        <v>59</v>
+        <v>110</v>
       </c>
       <c r="D27" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>59</v>
+        <v>107</v>
       </c>
       <c r="B28" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C28" t="s">
-        <v>59</v>
+        <v>111</v>
       </c>
       <c r="D28" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>39</v>
+        <v>107</v>
       </c>
       <c r="B29" t="s">
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="C29" t="s">
-        <v>39</v>
+        <v>112</v>
       </c>
       <c r="D29" t="s">
-        <v>22</v>
+        <v>69</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="B30" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="C30" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="D30" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>12</v>
+        <v>78</v>
       </c>
       <c r="B31" t="s">
-        <v>11</v>
+        <v>79</v>
       </c>
       <c r="C31" t="s">
-        <v>12</v>
+        <v>78</v>
       </c>
       <c r="D31" t="s">
-        <v>14</v>
+        <v>80</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>12</v>
+        <v>78</v>
       </c>
       <c r="B32" t="s">
-        <v>11</v>
+        <v>79</v>
       </c>
       <c r="C32" t="s">
-        <v>15</v>
+        <v>78</v>
       </c>
       <c r="D32" t="s">
-        <v>14</v>
+        <v>81</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>36</v>
+        <v>62</v>
       </c>
       <c r="B33" t="s">
-        <v>31</v>
+        <v>61</v>
       </c>
       <c r="C33" t="s">
-        <v>37</v>
+        <v>62</v>
       </c>
       <c r="D33" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="B34" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="C34" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="D34" t="s">
         <v>52</v>
@@ -1207,315 +1288,553 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>54</v>
+        <v>21</v>
       </c>
       <c r="B35" t="s">
-        <v>55</v>
+        <v>20</v>
       </c>
       <c r="C35" t="s">
-        <v>54</v>
+        <v>21</v>
       </c>
       <c r="D35" t="s">
-        <v>56</v>
+        <v>22</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="B36" t="s">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="C36" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="D36" t="s">
-        <v>2</v>
+        <v>23</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="B37" t="s">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="C37" t="s">
-        <v>1</v>
+        <v>38</v>
       </c>
       <c r="D37" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="B38" t="s">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="C38" t="s">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="D38" t="s">
-        <v>2</v>
+        <v>22</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="B39" t="s">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="C39" t="s">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="D39" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="B40" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C40" t="s">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="D40" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="B41" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="C41" t="s">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="D41" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>26</v>
+        <v>63</v>
       </c>
       <c r="B42" t="s">
-        <v>25</v>
+        <v>64</v>
       </c>
       <c r="C42" t="s">
-        <v>20</v>
+        <v>65</v>
       </c>
       <c r="D42" t="s">
-        <v>26</v>
+        <v>64</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>24</v>
+        <v>63</v>
       </c>
       <c r="B43" t="s">
-        <v>42</v>
+        <v>64</v>
       </c>
       <c r="C43" t="s">
-        <v>24</v>
+        <v>65</v>
       </c>
       <c r="D43" t="s">
-        <v>41</v>
+        <v>64</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="B44" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="C44" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="D44" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="B45" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="C45" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="D45" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="B46" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="C46" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="D46" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>82</v>
+        <v>39</v>
       </c>
       <c r="B47" t="s">
-        <v>83</v>
+        <v>20</v>
       </c>
       <c r="C47" t="s">
-        <v>82</v>
+        <v>39</v>
       </c>
       <c r="D47" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>82</v>
+        <v>12</v>
       </c>
       <c r="B48" t="s">
-        <v>83</v>
+        <v>11</v>
       </c>
       <c r="C48" t="s">
-        <v>82</v>
+        <v>12</v>
       </c>
       <c r="D48" t="s">
-        <v>84</v>
+        <v>13</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>85</v>
+        <v>12</v>
       </c>
       <c r="B49" t="s">
-        <v>86</v>
+        <v>11</v>
       </c>
       <c r="C49" t="s">
-        <v>85</v>
+        <v>12</v>
       </c>
       <c r="D49" t="s">
-        <v>87</v>
+        <v>14</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>89</v>
+        <v>12</v>
       </c>
       <c r="B50" t="s">
-        <v>90</v>
+        <v>11</v>
       </c>
       <c r="C50" t="s">
-        <v>89</v>
+        <v>15</v>
       </c>
       <c r="D50" t="s">
-        <v>88</v>
+        <v>14</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>89</v>
+        <v>36</v>
       </c>
       <c r="B51" t="s">
-        <v>90</v>
+        <v>31</v>
       </c>
       <c r="C51" t="s">
-        <v>89</v>
+        <v>37</v>
       </c>
       <c r="D51" t="s">
-        <v>91</v>
+        <v>31</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>92</v>
+        <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>79</v>
+        <v>52</v>
       </c>
       <c r="C52" t="s">
-        <v>92</v>
+        <v>53</v>
       </c>
       <c r="D52" t="s">
-        <v>81</v>
+        <v>52</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>92</v>
+        <v>54</v>
       </c>
       <c r="B53" t="s">
-        <v>79</v>
+        <v>55</v>
       </c>
       <c r="C53" t="s">
-        <v>92</v>
+        <v>54</v>
       </c>
       <c r="D53" t="s">
-        <v>80</v>
+        <v>56</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>93</v>
+        <v>3</v>
       </c>
       <c r="B54" t="s">
-        <v>86</v>
+        <v>0</v>
       </c>
       <c r="C54" t="s">
-        <v>93</v>
+        <v>1</v>
       </c>
       <c r="D54" t="s">
-        <v>94</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>63</v>
+        <v>3</v>
       </c>
       <c r="B55" t="s">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="C55" t="s">
-        <v>65</v>
+        <v>1</v>
       </c>
       <c r="D55" t="s">
-        <v>64</v>
+        <v>4</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
+        <v>3</v>
+      </c>
+      <c r="B56" t="s">
+        <v>0</v>
+      </c>
+      <c r="C56" t="s">
+        <v>3</v>
+      </c>
+      <c r="D56" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>3</v>
+      </c>
+      <c r="B57" t="s">
+        <v>0</v>
+      </c>
+      <c r="C57" t="s">
+        <v>3</v>
+      </c>
+      <c r="D57" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>89</v>
+      </c>
+      <c r="B58" t="s">
+        <v>90</v>
+      </c>
+      <c r="C58" t="s">
+        <v>89</v>
+      </c>
+      <c r="D58" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>89</v>
+      </c>
+      <c r="B59" t="s">
+        <v>90</v>
+      </c>
+      <c r="C59" t="s">
+        <v>89</v>
+      </c>
+      <c r="D59" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>8</v>
+      </c>
+      <c r="B60" t="s">
+        <v>10</v>
+      </c>
+      <c r="C60" t="s">
+        <v>9</v>
+      </c>
+      <c r="D60" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>44</v>
+      </c>
+      <c r="B61" t="s">
+        <v>43</v>
+      </c>
+      <c r="C61" t="s">
+        <v>44</v>
+      </c>
+      <c r="D61" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>92</v>
+      </c>
+      <c r="B62" t="s">
+        <v>79</v>
+      </c>
+      <c r="C62" t="s">
+        <v>92</v>
+      </c>
+      <c r="D62" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>92</v>
+      </c>
+      <c r="B63" t="s">
+        <v>79</v>
+      </c>
+      <c r="C63" t="s">
+        <v>92</v>
+      </c>
+      <c r="D63" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>26</v>
+      </c>
+      <c r="B64" t="s">
+        <v>25</v>
+      </c>
+      <c r="C64" t="s">
+        <v>20</v>
+      </c>
+      <c r="D64" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>24</v>
+      </c>
+      <c r="B65" t="s">
+        <v>42</v>
+      </c>
+      <c r="C65" t="s">
+        <v>24</v>
+      </c>
+      <c r="D65" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
         <v>96</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B66" t="s">
         <v>95</v>
       </c>
-      <c r="C56" t="s">
+      <c r="C66" t="s">
         <v>97</v>
       </c>
-      <c r="D56" t="s">
+      <c r="D66" t="s">
         <v>95</v>
       </c>
     </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>46</v>
+      </c>
+      <c r="B67" t="s">
+        <v>47</v>
+      </c>
+      <c r="C67" t="s">
+        <v>48</v>
+      </c>
+      <c r="D67" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>46</v>
+      </c>
+      <c r="B68" t="s">
+        <v>47</v>
+      </c>
+      <c r="C68" t="s">
+        <v>49</v>
+      </c>
+      <c r="D68" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>46</v>
+      </c>
+      <c r="B69" t="s">
+        <v>47</v>
+      </c>
+      <c r="C69" t="s">
+        <v>49</v>
+      </c>
+      <c r="D69" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>82</v>
+      </c>
+      <c r="B70" t="s">
+        <v>83</v>
+      </c>
+      <c r="C70" t="s">
+        <v>82</v>
+      </c>
+      <c r="D70" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>82</v>
+      </c>
+      <c r="B71" t="s">
+        <v>83</v>
+      </c>
+      <c r="C71" t="s">
+        <v>82</v>
+      </c>
+      <c r="D71" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>121</v>
+      </c>
+      <c r="B72" t="s">
+        <v>25</v>
+      </c>
+      <c r="C72" t="s">
+        <v>121</v>
+      </c>
+      <c r="D72" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>122</v>
+      </c>
+      <c r="B73" t="s">
+        <v>123</v>
+      </c>
+      <c r="C73" t="s">
+        <v>124</v>
+      </c>
+      <c r="D73" t="s">
+        <v>123</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D46">
-    <sortCondition ref="A2:A46"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D71">
+    <sortCondition ref="A2:A71"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
BM validation Jan 22
</commit_message>
<xml_diff>
--- a/src/inputs/canonical_nodes.xlsx
+++ b/src/inputs/canonical_nodes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ben/Documents/bruegel/data_new/WORKING/INDUSTRY/tuone_v6/src/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BF8E261-3391-7D4C-B64E-30505EE60E3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E13DC76B-05DD-2F45-B55F-D47A966FA5CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="16940" xr2:uid="{EBC50A8D-91C7-594D-A950-AF99F2B3F4AF}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="143">
   <si>
     <t>Pylon LifeEU</t>
   </si>
@@ -412,6 +412,60 @@
   </si>
   <si>
     <t>Arendal</t>
+  </si>
+  <si>
+    <t>Samsung</t>
+  </si>
+  <si>
+    <t>Gera</t>
+  </si>
+  <si>
+    <t>Gera-Cretzschwitz</t>
+  </si>
+  <si>
+    <t>Cologne</t>
+  </si>
+  <si>
+    <t>Cologne Merkenich</t>
+  </si>
+  <si>
+    <t>Ford</t>
+  </si>
+  <si>
+    <t>Langen</t>
+  </si>
+  <si>
+    <t>Akasol</t>
+  </si>
+  <si>
+    <t>Darmstadt</t>
+  </si>
+  <si>
+    <t>Dolnośląskie</t>
+  </si>
+  <si>
+    <t>Wroclaw</t>
+  </si>
+  <si>
+    <t>Customcells</t>
+  </si>
+  <si>
+    <t>Tübingen</t>
+  </si>
+  <si>
+    <t>Cellforce</t>
+  </si>
+  <si>
+    <t>Kaiserslautern</t>
+  </si>
+  <si>
+    <t>Opel</t>
+  </si>
+  <si>
+    <t>PSA Group</t>
+  </si>
+  <si>
+    <t>Saft</t>
   </si>
 </sst>
 </file>
@@ -799,7 +853,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DF9B3CA-7DC7-BB45-882F-C1DDB5BD93A3}">
-  <dimension ref="A1:E73"/>
+  <dimension ref="A1:E83"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.5" bestFit="1" customWidth="1"/>
@@ -1820,16 +1874,156 @@
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B73" t="s">
         <v>123</v>
       </c>
       <c r="C73" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D73" t="s">
         <v>123</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>127</v>
+      </c>
+      <c r="B74" t="s">
+        <v>125</v>
+      </c>
+      <c r="C74" t="s">
+        <v>126</v>
+      </c>
+      <c r="D74" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>128</v>
+      </c>
+      <c r="B75" t="s">
+        <v>130</v>
+      </c>
+      <c r="C75" t="s">
+        <v>129</v>
+      </c>
+      <c r="D75" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
+        <v>131</v>
+      </c>
+      <c r="B76" t="s">
+        <v>132</v>
+      </c>
+      <c r="C76" t="s">
+        <v>133</v>
+      </c>
+      <c r="D76" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>134</v>
+      </c>
+      <c r="B77" t="s">
+        <v>56</v>
+      </c>
+      <c r="C77" t="s">
+        <v>135</v>
+      </c>
+      <c r="D77" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>137</v>
+      </c>
+      <c r="B78" t="s">
+        <v>136</v>
+      </c>
+      <c r="C78" t="s">
+        <v>137</v>
+      </c>
+      <c r="D78" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
+        <v>137</v>
+      </c>
+      <c r="B79" t="s">
+        <v>136</v>
+      </c>
+      <c r="C79" t="s">
+        <v>137</v>
+      </c>
+      <c r="D79" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
+        <v>139</v>
+      </c>
+      <c r="B80" t="s">
+        <v>25</v>
+      </c>
+      <c r="C80" t="s">
+        <v>139</v>
+      </c>
+      <c r="D80" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
+        <v>139</v>
+      </c>
+      <c r="B81" t="s">
+        <v>25</v>
+      </c>
+      <c r="C81" t="s">
+        <v>139</v>
+      </c>
+      <c r="D81" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>139</v>
+      </c>
+      <c r="B82" t="s">
+        <v>25</v>
+      </c>
+      <c r="C82" t="s">
+        <v>139</v>
+      </c>
+      <c r="D82" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>139</v>
+      </c>
+      <c r="B83" t="s">
+        <v>25</v>
+      </c>
+      <c r="C83" t="s">
+        <v>139</v>
+      </c>
+      <c r="D83" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Stop tracking .obsidian folder and resolved .DS_Store conflict
</commit_message>
<xml_diff>
--- a/src/inputs/canonical_nodes.xlsx
+++ b/src/inputs/canonical_nodes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10112"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ben/Documents/bruegel/data_new/WORKING/INDUSTRY/tuone_v6/src/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FF8F43F-F347-5847-91CC-152141D5BF11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{542A4A1B-98E6-B444-B483-A8838E81452E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="16940" xr2:uid="{EBC50A8D-91C7-594D-A950-AF99F2B3F4AF}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="175">
   <si>
     <t>Pylon LifeEU</t>
   </si>
@@ -466,6 +466,102 @@
   </si>
   <si>
     <t>Saft</t>
+  </si>
+  <si>
+    <t>Freyr</t>
+  </si>
+  <si>
+    <t>Mo i Rana</t>
+  </si>
+  <si>
+    <t>Giga Arctic</t>
+  </si>
+  <si>
+    <t>Döbeln</t>
+  </si>
+  <si>
+    <t>Blackstone Resources</t>
+  </si>
+  <si>
+    <t>Saxony</t>
+  </si>
+  <si>
+    <t>Chemnitz</t>
+  </si>
+  <si>
+    <t>Baden-Württemberg</t>
+  </si>
+  <si>
+    <t>Envision AESC</t>
+  </si>
+  <si>
+    <t>Douai</t>
+  </si>
+  <si>
+    <t>AESC</t>
+  </si>
+  <si>
+    <t>AESC Envision</t>
+  </si>
+  <si>
+    <t>AESC-Envision</t>
+  </si>
+  <si>
+    <t>Verkor</t>
+  </si>
+  <si>
+    <t>Dunkirk</t>
+  </si>
+  <si>
+    <t>Recharge Industries</t>
+  </si>
+  <si>
+    <t>Sunderland</t>
+  </si>
+  <si>
+    <t>Gotion InoBat Batteries</t>
+  </si>
+  <si>
+    <t>Šurany</t>
+  </si>
+  <si>
+    <t>InoBat Auto</t>
+  </si>
+  <si>
+    <t>Gotion High-Tech</t>
+  </si>
+  <si>
+    <t>Göd</t>
+  </si>
+  <si>
+    <t>Budapest</t>
+  </si>
+  <si>
+    <t>Valmet</t>
+  </si>
+  <si>
+    <t>Kirchardt</t>
+  </si>
+  <si>
+    <t>Bad Friedrichshall</t>
+  </si>
+  <si>
+    <t>Heilbronn</t>
+  </si>
+  <si>
+    <t>Kirchhardt</t>
+  </si>
+  <si>
+    <t>Weihenbronn</t>
+  </si>
+  <si>
+    <t>Chasseneuil-du-Poitou</t>
+  </si>
+  <si>
+    <t>Poitiers</t>
+  </si>
+  <si>
+    <t>Forsee Power</t>
   </si>
 </sst>
 </file>
@@ -853,13 +949,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DF9B3CA-7DC7-BB45-882F-C1DDB5BD93A3}">
-  <dimension ref="A1:E83"/>
+  <dimension ref="A1:E100"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.1640625" customWidth="1"/>
     <col min="3" max="3" width="36.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.1640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
   </cols>
   <sheetData>
@@ -894,44 +990,44 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>124</v>
       </c>
       <c r="B3" t="s">
-        <v>28</v>
+        <v>123</v>
       </c>
       <c r="C3" t="s">
-        <v>29</v>
+        <v>122</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>76</v>
+        <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s">
-        <v>76</v>
+        <v>29</v>
       </c>
       <c r="D4" t="s">
-        <v>77</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>113</v>
+        <v>76</v>
       </c>
       <c r="B5" t="s">
-        <v>114</v>
+        <v>75</v>
       </c>
       <c r="C5" t="s">
-        <v>115</v>
+        <v>76</v>
       </c>
       <c r="D5" t="s">
-        <v>114</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -942,7 +1038,7 @@
         <v>114</v>
       </c>
       <c r="C6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D6" t="s">
         <v>114</v>
@@ -950,72 +1046,72 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="B7" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="C7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D7" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="B8" t="s">
-        <v>119</v>
+        <v>158</v>
       </c>
       <c r="C8" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D8" t="s">
-        <v>119</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>85</v>
+        <v>118</v>
       </c>
       <c r="B9" t="s">
-        <v>86</v>
+        <v>119</v>
       </c>
       <c r="C9" t="s">
-        <v>85</v>
+        <v>117</v>
       </c>
       <c r="D9" t="s">
-        <v>87</v>
+        <v>119</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>30</v>
+        <v>118</v>
       </c>
       <c r="B10" t="s">
-        <v>31</v>
+        <v>119</v>
       </c>
       <c r="C10" t="s">
-        <v>32</v>
+        <v>120</v>
       </c>
       <c r="D10" t="s">
-        <v>31</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>30</v>
+        <v>85</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
+        <v>86</v>
       </c>
       <c r="C11" t="s">
-        <v>32</v>
+        <v>85</v>
       </c>
       <c r="D11" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
@@ -1026,10 +1122,10 @@
         <v>31</v>
       </c>
       <c r="C12" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D12" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
@@ -1040,10 +1136,10 @@
         <v>31</v>
       </c>
       <c r="C13" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D13" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
@@ -1057,978 +1153,1216 @@
         <v>30</v>
       </c>
       <c r="D14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>98</v>
+        <v>30</v>
       </c>
       <c r="B15" t="s">
-        <v>99</v>
+        <v>31</v>
       </c>
       <c r="C15" t="s">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="D15" t="s">
-        <v>99</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>101</v>
+        <v>30</v>
       </c>
       <c r="B16" t="s">
-        <v>84</v>
+        <v>31</v>
       </c>
       <c r="C16" t="s">
-        <v>102</v>
+        <v>30</v>
       </c>
       <c r="D16" t="s">
-        <v>84</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>101</v>
+        <v>128</v>
       </c>
       <c r="B17" t="s">
-        <v>84</v>
+        <v>130</v>
       </c>
       <c r="C17" t="s">
-        <v>103</v>
+        <v>129</v>
       </c>
       <c r="D17" t="s">
-        <v>84</v>
+        <v>130</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B18" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="C18" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D18" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>67</v>
+        <v>146</v>
       </c>
       <c r="B19" t="s">
-        <v>66</v>
+        <v>147</v>
       </c>
       <c r="C19" t="s">
-        <v>67</v>
+        <v>148</v>
       </c>
       <c r="D19" t="s">
-        <v>68</v>
+        <v>147</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>146</v>
       </c>
       <c r="B20" t="s">
-        <v>71</v>
+        <v>147</v>
       </c>
       <c r="C20" t="s">
-        <v>70</v>
+        <v>149</v>
       </c>
       <c r="D20" t="s">
-        <v>72</v>
+        <v>147</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>70</v>
+        <v>134</v>
       </c>
       <c r="B21" t="s">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="C21" t="s">
-        <v>70</v>
+        <v>135</v>
       </c>
       <c r="D21" t="s">
-        <v>73</v>
+        <v>56</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>70</v>
+        <v>152</v>
       </c>
       <c r="B22" t="s">
-        <v>71</v>
+        <v>151</v>
       </c>
       <c r="C22" t="s">
-        <v>70</v>
+        <v>152</v>
       </c>
       <c r="D22" t="s">
-        <v>74</v>
+        <v>153</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>107</v>
+        <v>152</v>
       </c>
       <c r="B23" t="s">
-        <v>69</v>
+        <v>151</v>
       </c>
       <c r="C23" t="s">
-        <v>106</v>
+        <v>152</v>
       </c>
       <c r="D23" t="s">
-        <v>69</v>
+        <v>154</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>107</v>
+        <v>152</v>
       </c>
       <c r="B24" t="s">
-        <v>69</v>
+        <v>151</v>
       </c>
       <c r="C24" t="s">
-        <v>105</v>
+        <v>152</v>
       </c>
       <c r="D24" t="s">
-        <v>69</v>
+        <v>155</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="B25" t="s">
-        <v>69</v>
+        <v>25</v>
       </c>
       <c r="C25" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="D25" t="s">
-        <v>69</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>107</v>
+        <v>157</v>
       </c>
       <c r="B26" t="s">
-        <v>69</v>
+        <v>156</v>
       </c>
       <c r="C26" t="s">
-        <v>109</v>
+        <v>152</v>
       </c>
       <c r="D26" t="s">
-        <v>69</v>
+        <v>156</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="B27" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="C27" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="D27" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="B28" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="C28" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="D28" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="B29" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="C29" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="D29" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>5</v>
+        <v>127</v>
       </c>
       <c r="B30" t="s">
-        <v>6</v>
+        <v>125</v>
       </c>
       <c r="C30" t="s">
-        <v>5</v>
+        <v>126</v>
       </c>
       <c r="D30" t="s">
-        <v>7</v>
+        <v>125</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="B31" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="C31" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="D31" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="B32" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="C32" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="D32" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="B33" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="C33" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="D33" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="B34" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="C34" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="D34" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>21</v>
+        <v>107</v>
       </c>
       <c r="B35" t="s">
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="C35" t="s">
-        <v>21</v>
+        <v>106</v>
       </c>
       <c r="D35" t="s">
-        <v>22</v>
+        <v>69</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>21</v>
+        <v>107</v>
       </c>
       <c r="B36" t="s">
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="C36" t="s">
-        <v>21</v>
+        <v>105</v>
       </c>
       <c r="D36" t="s">
-        <v>23</v>
+        <v>69</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>21</v>
+        <v>107</v>
       </c>
       <c r="B37" t="s">
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="C37" t="s">
-        <v>38</v>
+        <v>108</v>
       </c>
       <c r="D37" t="s">
-        <v>22</v>
+        <v>69</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>21</v>
+        <v>107</v>
       </c>
       <c r="B38" t="s">
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="C38" t="s">
-        <v>24</v>
+        <v>109</v>
       </c>
       <c r="D38" t="s">
-        <v>22</v>
+        <v>69</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>21</v>
+        <v>107</v>
       </c>
       <c r="B39" t="s">
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="C39" t="s">
-        <v>24</v>
+        <v>110</v>
       </c>
       <c r="D39" t="s">
-        <v>23</v>
+        <v>69</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>21</v>
+        <v>107</v>
       </c>
       <c r="B40" t="s">
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="C40" t="s">
-        <v>24</v>
+        <v>111</v>
       </c>
       <c r="D40" t="s">
-        <v>20</v>
+        <v>69</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>21</v>
+        <v>107</v>
       </c>
       <c r="B41" t="s">
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="C41" t="s">
-        <v>24</v>
+        <v>112</v>
       </c>
       <c r="D41" t="s">
-        <v>40</v>
+        <v>69</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>63</v>
+        <v>139</v>
       </c>
       <c r="B42" t="s">
-        <v>64</v>
+        <v>25</v>
       </c>
       <c r="C42" t="s">
-        <v>65</v>
+        <v>139</v>
       </c>
       <c r="D42" t="s">
-        <v>64</v>
+        <v>140</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>63</v>
+        <v>139</v>
       </c>
       <c r="B43" t="s">
-        <v>64</v>
+        <v>25</v>
       </c>
       <c r="C43" t="s">
-        <v>65</v>
+        <v>139</v>
       </c>
       <c r="D43" t="s">
-        <v>64</v>
+        <v>141</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>57</v>
+        <v>139</v>
       </c>
       <c r="B44" t="s">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="C44" t="s">
-        <v>57</v>
+        <v>139</v>
       </c>
       <c r="D44" t="s">
-        <v>58</v>
+        <v>142</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>59</v>
+        <v>139</v>
       </c>
       <c r="B45" t="s">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="C45" t="s">
-        <v>59</v>
+        <v>139</v>
       </c>
       <c r="D45" t="s">
-        <v>58</v>
+        <v>20</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>59</v>
+        <v>131</v>
       </c>
       <c r="B46" t="s">
-        <v>52</v>
+        <v>132</v>
       </c>
       <c r="C46" t="s">
-        <v>59</v>
+        <v>133</v>
       </c>
       <c r="D46" t="s">
-        <v>60</v>
+        <v>132</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="B47" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="C47" t="s">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="D47" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>12</v>
+        <v>78</v>
       </c>
       <c r="B48" t="s">
-        <v>11</v>
+        <v>79</v>
       </c>
       <c r="C48" t="s">
-        <v>12</v>
+        <v>78</v>
       </c>
       <c r="D48" t="s">
-        <v>13</v>
+        <v>80</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>12</v>
+        <v>78</v>
       </c>
       <c r="B49" t="s">
-        <v>11</v>
+        <v>79</v>
       </c>
       <c r="C49" t="s">
-        <v>12</v>
+        <v>78</v>
       </c>
       <c r="D49" t="s">
-        <v>14</v>
+        <v>81</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="B50" t="s">
-        <v>11</v>
+        <v>61</v>
       </c>
       <c r="C50" t="s">
-        <v>15</v>
+        <v>62</v>
       </c>
       <c r="D50" t="s">
-        <v>14</v>
+        <v>60</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>36</v>
+        <v>62</v>
       </c>
       <c r="B51" t="s">
-        <v>31</v>
+        <v>61</v>
       </c>
       <c r="C51" t="s">
-        <v>37</v>
+        <v>62</v>
       </c>
       <c r="D51" t="s">
-        <v>31</v>
+        <v>52</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>51</v>
+        <v>21</v>
       </c>
       <c r="B52" t="s">
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="C52" t="s">
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="D52" t="s">
-        <v>52</v>
+        <v>22</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>54</v>
+        <v>21</v>
       </c>
       <c r="B53" t="s">
-        <v>55</v>
+        <v>20</v>
       </c>
       <c r="C53" t="s">
-        <v>54</v>
+        <v>21</v>
       </c>
       <c r="D53" t="s">
-        <v>56</v>
+        <v>23</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="B54" t="s">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="C54" t="s">
-        <v>1</v>
+        <v>38</v>
       </c>
       <c r="D54" t="s">
-        <v>2</v>
+        <v>22</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="B55" t="s">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="C55" t="s">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="D55" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="B56" t="s">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="C56" t="s">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="D56" t="s">
-        <v>2</v>
+        <v>23</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="B57" t="s">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="C57" t="s">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="D57" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>89</v>
+        <v>21</v>
       </c>
       <c r="B58" t="s">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="C58" t="s">
-        <v>89</v>
+        <v>24</v>
       </c>
       <c r="D58" t="s">
-        <v>88</v>
+        <v>40</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>89</v>
+        <v>144</v>
       </c>
       <c r="B59" t="s">
-        <v>90</v>
+        <v>143</v>
       </c>
       <c r="C59" t="s">
-        <v>89</v>
+        <v>145</v>
       </c>
       <c r="D59" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>8</v>
+        <v>63</v>
       </c>
       <c r="B60" t="s">
-        <v>10</v>
+        <v>64</v>
       </c>
       <c r="C60" t="s">
-        <v>9</v>
+        <v>65</v>
       </c>
       <c r="D60" t="s">
-        <v>10</v>
+        <v>64</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="B61" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="C61" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="D61" t="s">
-        <v>45</v>
+        <v>64</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>92</v>
+        <v>57</v>
       </c>
       <c r="B62" t="s">
-        <v>79</v>
+        <v>52</v>
       </c>
       <c r="C62" t="s">
-        <v>92</v>
+        <v>57</v>
       </c>
       <c r="D62" t="s">
-        <v>81</v>
+        <v>58</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>92</v>
+        <v>59</v>
       </c>
       <c r="B63" t="s">
-        <v>79</v>
+        <v>52</v>
       </c>
       <c r="C63" t="s">
-        <v>92</v>
+        <v>59</v>
       </c>
       <c r="D63" t="s">
-        <v>80</v>
+        <v>58</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>26</v>
+        <v>59</v>
       </c>
       <c r="B64" t="s">
-        <v>25</v>
+        <v>52</v>
       </c>
       <c r="C64" t="s">
-        <v>20</v>
+        <v>59</v>
       </c>
       <c r="D64" t="s">
-        <v>26</v>
+        <v>60</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="B65" t="s">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="C65" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="D65" t="s">
-        <v>41</v>
+        <v>22</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>96</v>
+        <v>12</v>
       </c>
       <c r="B66" t="s">
-        <v>95</v>
+        <v>11</v>
       </c>
       <c r="C66" t="s">
-        <v>97</v>
+        <v>12</v>
       </c>
       <c r="D66" t="s">
-        <v>95</v>
+        <v>13</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="B67" t="s">
-        <v>47</v>
+        <v>11</v>
       </c>
       <c r="C67" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="D67" t="s">
-        <v>47</v>
+        <v>14</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="B68" t="s">
-        <v>47</v>
+        <v>11</v>
       </c>
       <c r="C68" t="s">
-        <v>49</v>
+        <v>15</v>
       </c>
       <c r="D68" t="s">
-        <v>47</v>
+        <v>14</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="B69" t="s">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="C69" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="D69" t="s">
-        <v>50</v>
+        <v>31</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>82</v>
+        <v>51</v>
       </c>
       <c r="B70" t="s">
-        <v>83</v>
+        <v>52</v>
       </c>
       <c r="C70" t="s">
-        <v>82</v>
+        <v>53</v>
       </c>
       <c r="D70" t="s">
-        <v>20</v>
+        <v>52</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>82</v>
+        <v>54</v>
       </c>
       <c r="B71" t="s">
-        <v>83</v>
+        <v>55</v>
       </c>
       <c r="C71" t="s">
-        <v>82</v>
+        <v>54</v>
       </c>
       <c r="D71" t="s">
-        <v>84</v>
+        <v>56</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>121</v>
+        <v>3</v>
       </c>
       <c r="B72" t="s">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="C72" t="s">
-        <v>121</v>
+        <v>1</v>
       </c>
       <c r="D72" t="s">
-        <v>20</v>
+        <v>2</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>124</v>
+        <v>3</v>
       </c>
       <c r="B73" t="s">
-        <v>123</v>
+        <v>0</v>
       </c>
       <c r="C73" t="s">
-        <v>122</v>
+        <v>1</v>
       </c>
       <c r="D73" t="s">
-        <v>123</v>
+        <v>4</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>127</v>
+        <v>3</v>
       </c>
       <c r="B74" t="s">
-        <v>125</v>
+        <v>0</v>
       </c>
       <c r="C74" t="s">
-        <v>126</v>
+        <v>3</v>
       </c>
       <c r="D74" t="s">
-        <v>125</v>
+        <v>2</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>128</v>
+        <v>3</v>
       </c>
       <c r="B75" t="s">
-        <v>130</v>
+        <v>0</v>
       </c>
       <c r="C75" t="s">
-        <v>129</v>
+        <v>3</v>
       </c>
       <c r="D75" t="s">
-        <v>130</v>
+        <v>4</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>131</v>
+        <v>89</v>
       </c>
       <c r="B76" t="s">
-        <v>132</v>
+        <v>90</v>
       </c>
       <c r="C76" t="s">
-        <v>133</v>
+        <v>89</v>
       </c>
       <c r="D76" t="s">
-        <v>132</v>
+        <v>88</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>134</v>
+        <v>89</v>
       </c>
       <c r="B77" t="s">
-        <v>56</v>
+        <v>90</v>
       </c>
       <c r="C77" t="s">
-        <v>135</v>
+        <v>89</v>
       </c>
       <c r="D77" t="s">
-        <v>56</v>
+        <v>91</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>137</v>
+        <v>8</v>
       </c>
       <c r="B78" t="s">
-        <v>136</v>
+        <v>10</v>
       </c>
       <c r="C78" t="s">
-        <v>137</v>
+        <v>9</v>
       </c>
       <c r="D78" t="s">
-        <v>138</v>
+        <v>10</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>137</v>
+        <v>44</v>
       </c>
       <c r="B79" t="s">
-        <v>136</v>
+        <v>43</v>
       </c>
       <c r="C79" t="s">
-        <v>137</v>
+        <v>44</v>
       </c>
       <c r="D79" t="s">
-        <v>74</v>
+        <v>45</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>139</v>
+        <v>159</v>
       </c>
       <c r="B80" t="s">
-        <v>25</v>
+        <v>151</v>
       </c>
       <c r="C80" t="s">
-        <v>139</v>
+        <v>159</v>
       </c>
       <c r="D80" t="s">
-        <v>140</v>
+        <v>154</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>139</v>
+        <v>92</v>
       </c>
       <c r="B81" t="s">
-        <v>25</v>
+        <v>79</v>
       </c>
       <c r="C81" t="s">
-        <v>139</v>
+        <v>92</v>
       </c>
       <c r="D81" t="s">
-        <v>141</v>
+        <v>81</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>139</v>
+        <v>92</v>
       </c>
       <c r="B82" t="s">
-        <v>25</v>
+        <v>79</v>
       </c>
       <c r="C82" t="s">
-        <v>139</v>
+        <v>92</v>
       </c>
       <c r="D82" t="s">
-        <v>142</v>
+        <v>80</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>139</v>
+        <v>26</v>
       </c>
       <c r="B83" t="s">
         <v>25</v>
       </c>
       <c r="C83" t="s">
-        <v>139</v>
+        <v>20</v>
       </c>
       <c r="D83" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
+        <v>137</v>
+      </c>
+      <c r="B84" t="s">
+        <v>136</v>
+      </c>
+      <c r="C84" t="s">
+        <v>137</v>
+      </c>
+      <c r="D84" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
+        <v>137</v>
+      </c>
+      <c r="B85" t="s">
+        <v>136</v>
+      </c>
+      <c r="C85" t="s">
+        <v>137</v>
+      </c>
+      <c r="D85" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
+        <v>137</v>
+      </c>
+      <c r="B86" t="s">
+        <v>136</v>
+      </c>
+      <c r="C86" t="s">
+        <v>150</v>
+      </c>
+      <c r="D86" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>24</v>
+      </c>
+      <c r="B87" t="s">
+        <v>42</v>
+      </c>
+      <c r="C87" t="s">
+        <v>24</v>
+      </c>
+      <c r="D87" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>96</v>
+      </c>
+      <c r="B88" t="s">
+        <v>95</v>
+      </c>
+      <c r="C88" t="s">
+        <v>97</v>
+      </c>
+      <c r="D88" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>46</v>
+      </c>
+      <c r="B89" t="s">
+        <v>47</v>
+      </c>
+      <c r="C89" t="s">
+        <v>48</v>
+      </c>
+      <c r="D89" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>46</v>
+      </c>
+      <c r="B90" t="s">
+        <v>47</v>
+      </c>
+      <c r="C90" t="s">
+        <v>49</v>
+      </c>
+      <c r="D90" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>46</v>
+      </c>
+      <c r="B91" t="s">
+        <v>47</v>
+      </c>
+      <c r="C91" t="s">
+        <v>49</v>
+      </c>
+      <c r="D91" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>82</v>
+      </c>
+      <c r="B92" t="s">
+        <v>83</v>
+      </c>
+      <c r="C92" t="s">
+        <v>82</v>
+      </c>
+      <c r="D92" t="s">
         <v>20</v>
       </c>
     </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>82</v>
+      </c>
+      <c r="B93" t="s">
+        <v>83</v>
+      </c>
+      <c r="C93" t="s">
+        <v>82</v>
+      </c>
+      <c r="D93" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
+        <v>161</v>
+      </c>
+      <c r="B94" t="s">
+        <v>160</v>
+      </c>
+      <c r="C94" t="s">
+        <v>161</v>
+      </c>
+      <c r="D94" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
+        <v>161</v>
+      </c>
+      <c r="B95" t="s">
+        <v>160</v>
+      </c>
+      <c r="C95" t="s">
+        <v>161</v>
+      </c>
+      <c r="D95" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A96" t="s">
+        <v>164</v>
+      </c>
+      <c r="B96" t="s">
+        <v>125</v>
+      </c>
+      <c r="C96" t="s">
+        <v>165</v>
+      </c>
+      <c r="D96" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A97" t="s">
+        <v>167</v>
+      </c>
+      <c r="B97" t="s">
+        <v>166</v>
+      </c>
+      <c r="C97" t="s">
+        <v>169</v>
+      </c>
+      <c r="D97" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A98" t="s">
+        <v>167</v>
+      </c>
+      <c r="B98" t="s">
+        <v>166</v>
+      </c>
+      <c r="C98" t="s">
+        <v>170</v>
+      </c>
+      <c r="D98" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A99" t="s">
+        <v>168</v>
+      </c>
+      <c r="B99" t="s">
+        <v>166</v>
+      </c>
+      <c r="C99" t="s">
+        <v>171</v>
+      </c>
+      <c r="D99" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A100" t="s">
+        <v>173</v>
+      </c>
+      <c r="B100" t="s">
+        <v>174</v>
+      </c>
+      <c r="C100" t="s">
+        <v>172</v>
+      </c>
+      <c r="D100" t="s">
+        <v>174</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D71">
-    <sortCondition ref="A2:A71"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D93">
+    <sortCondition ref="A2:A93"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
validated battery cell projects from 200 to 180
</commit_message>
<xml_diff>
--- a/src/inputs/canonical_nodes.xlsx
+++ b/src/inputs/canonical_nodes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ben/Documents/bruegel/data_new/WORKING/INDUSTRY/tuone_v6/src/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{542A4A1B-98E6-B444-B483-A8838E81452E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8FB7FDF-8281-5849-90E6-0847217F9230}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="16940" xr2:uid="{EBC50A8D-91C7-594D-A950-AF99F2B3F4AF}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="184">
   <si>
     <t>Pylon LifeEU</t>
   </si>
@@ -562,6 +562,33 @@
   </si>
   <si>
     <t>Forsee Power</t>
+  </si>
+  <si>
+    <t>Navalmoral de la Mata</t>
+  </si>
+  <si>
+    <t>EMR</t>
+  </si>
+  <si>
+    <t>Hamburg</t>
+  </si>
+  <si>
+    <t>Heide</t>
+  </si>
+  <si>
+    <t>Schleswig-Holstein</t>
+  </si>
+  <si>
+    <t>Northvolt Ett</t>
+  </si>
+  <si>
+    <t>Skellefteå</t>
+  </si>
+  <si>
+    <t>Northvolt Ett gigafactory</t>
+  </si>
+  <si>
+    <t>Revolt Ett</t>
   </si>
 </sst>
 </file>
@@ -949,7 +976,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DF9B3CA-7DC7-BB45-882F-C1DDB5BD93A3}">
-  <dimension ref="A1:E100"/>
+  <dimension ref="A1:E106"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.5" bestFit="1" customWidth="1"/>
@@ -2358,6 +2385,90 @@
       </c>
       <c r="D100" t="s">
         <v>174</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A101" t="s">
+        <v>175</v>
+      </c>
+      <c r="B101" t="s">
+        <v>154</v>
+      </c>
+      <c r="C101" t="s">
+        <v>175</v>
+      </c>
+      <c r="D101" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A102" t="s">
+        <v>177</v>
+      </c>
+      <c r="B102" t="s">
+        <v>176</v>
+      </c>
+      <c r="C102" t="s">
+        <v>177</v>
+      </c>
+      <c r="D102" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A103" t="s">
+        <v>178</v>
+      </c>
+      <c r="B103" t="s">
+        <v>45</v>
+      </c>
+      <c r="C103" t="s">
+        <v>179</v>
+      </c>
+      <c r="D103" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A104" t="s">
+        <v>181</v>
+      </c>
+      <c r="B104" t="s">
+        <v>45</v>
+      </c>
+      <c r="C104" t="s">
+        <v>180</v>
+      </c>
+      <c r="D104" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A105" t="s">
+        <v>181</v>
+      </c>
+      <c r="B105" t="s">
+        <v>45</v>
+      </c>
+      <c r="C105" t="s">
+        <v>182</v>
+      </c>
+      <c r="D105" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A106" t="s">
+        <v>181</v>
+      </c>
+      <c r="B106" t="s">
+        <v>45</v>
+      </c>
+      <c r="C106" t="s">
+        <v>183</v>
+      </c>
+      <c r="D106" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
validated battery cell projects down to 120 left
</commit_message>
<xml_diff>
--- a/src/inputs/canonical_nodes.xlsx
+++ b/src/inputs/canonical_nodes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ben/Documents/bruegel/data_new/WORKING/INDUSTRY/tuone_v6/src/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8FB7FDF-8281-5849-90E6-0847217F9230}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC66DA15-3975-9344-B602-2A8F86A450A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="16940" xr2:uid="{EBC50A8D-91C7-594D-A950-AF99F2B3F4AF}"/>
+    <workbookView xWindow="0" yWindow="720" windowWidth="29400" windowHeight="16940" xr2:uid="{EBC50A8D-91C7-594D-A950-AF99F2B3F4AF}"/>
   </bookViews>
   <sheets>
     <sheet name="merge" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="195">
   <si>
     <t>Pylon LifeEU</t>
   </si>
@@ -589,6 +589,39 @@
   </si>
   <si>
     <t>Revolt Ett</t>
+  </si>
+  <si>
+    <t>Ett</t>
+  </si>
+  <si>
+    <t>Nersac</t>
+  </si>
+  <si>
+    <t>Umeå</t>
+  </si>
+  <si>
+    <t>Reutlingen</t>
+  </si>
+  <si>
+    <t>Valencia</t>
+  </si>
+  <si>
+    <t>Kobierzyce</t>
+  </si>
+  <si>
+    <t>Trnava</t>
+  </si>
+  <si>
+    <t>Untertürkheim Hedelfingen</t>
+  </si>
+  <si>
+    <t>Untertürkheim</t>
+  </si>
+  <si>
+    <t>Unterkücken</t>
+  </si>
+  <si>
+    <t>Mercedes-Benz</t>
   </si>
 </sst>
 </file>
@@ -976,7 +1009,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DF9B3CA-7DC7-BB45-882F-C1DDB5BD93A3}">
-  <dimension ref="A1:E106"/>
+  <dimension ref="A1:E119"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.5" bestFit="1" customWidth="1"/>
@@ -2109,16 +2142,16 @@
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>92</v>
+        <v>159</v>
       </c>
       <c r="B81" t="s">
-        <v>79</v>
+        <v>151</v>
       </c>
       <c r="C81" t="s">
-        <v>92</v>
+        <v>159</v>
       </c>
       <c r="D81" t="s">
-        <v>81</v>
+        <v>153</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.2">
@@ -2132,119 +2165,119 @@
         <v>92</v>
       </c>
       <c r="D82" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>26</v>
+        <v>92</v>
       </c>
       <c r="B83" t="s">
-        <v>25</v>
+        <v>79</v>
       </c>
       <c r="C83" t="s">
-        <v>20</v>
+        <v>92</v>
       </c>
       <c r="D83" t="s">
-        <v>26</v>
+        <v>80</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>137</v>
+        <v>26</v>
       </c>
       <c r="B84" t="s">
-        <v>136</v>
+        <v>25</v>
       </c>
       <c r="C84" t="s">
-        <v>137</v>
+        <v>20</v>
       </c>
       <c r="D84" t="s">
-        <v>138</v>
+        <v>26</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>137</v>
+        <v>187</v>
       </c>
       <c r="B85" t="s">
-        <v>136</v>
+        <v>74</v>
       </c>
       <c r="C85" t="s">
         <v>137</v>
       </c>
       <c r="D85" t="s">
-        <v>74</v>
+        <v>138</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
+        <v>187</v>
+      </c>
+      <c r="B86" t="s">
+        <v>74</v>
+      </c>
+      <c r="C86" t="s">
         <v>137</v>
       </c>
-      <c r="B86" t="s">
-        <v>136</v>
-      </c>
-      <c r="C86" t="s">
-        <v>150</v>
-      </c>
       <c r="D86" t="s">
-        <v>138</v>
+        <v>74</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>24</v>
+        <v>187</v>
       </c>
       <c r="B87" t="s">
-        <v>42</v>
+        <v>74</v>
       </c>
       <c r="C87" t="s">
-        <v>24</v>
+        <v>150</v>
       </c>
       <c r="D87" t="s">
-        <v>41</v>
+        <v>138</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>96</v>
+        <v>187</v>
       </c>
       <c r="B88" t="s">
-        <v>95</v>
+        <v>74</v>
       </c>
       <c r="C88" t="s">
-        <v>97</v>
+        <v>137</v>
       </c>
       <c r="D88" t="s">
-        <v>95</v>
+        <v>136</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>46</v>
+        <v>24</v>
       </c>
       <c r="B89" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C89" t="s">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="D89" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>46</v>
+        <v>96</v>
       </c>
       <c r="B90" t="s">
-        <v>47</v>
+        <v>95</v>
       </c>
       <c r="C90" t="s">
-        <v>49</v>
+        <v>97</v>
       </c>
       <c r="D90" t="s">
-        <v>47</v>
+        <v>95</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.2">
@@ -2255,119 +2288,119 @@
         <v>47</v>
       </c>
       <c r="C91" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D91" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>82</v>
+        <v>46</v>
       </c>
       <c r="B92" t="s">
-        <v>83</v>
+        <v>47</v>
       </c>
       <c r="C92" t="s">
-        <v>82</v>
+        <v>49</v>
       </c>
       <c r="D92" t="s">
-        <v>20</v>
+        <v>47</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>82</v>
+        <v>46</v>
       </c>
       <c r="B93" t="s">
-        <v>83</v>
+        <v>47</v>
       </c>
       <c r="C93" t="s">
-        <v>82</v>
+        <v>49</v>
       </c>
       <c r="D93" t="s">
-        <v>84</v>
+        <v>50</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>161</v>
+        <v>82</v>
       </c>
       <c r="B94" t="s">
-        <v>160</v>
+        <v>83</v>
       </c>
       <c r="C94" t="s">
-        <v>161</v>
+        <v>82</v>
       </c>
       <c r="D94" t="s">
-        <v>162</v>
+        <v>20</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>161</v>
+        <v>82</v>
       </c>
       <c r="B95" t="s">
-        <v>160</v>
+        <v>83</v>
       </c>
       <c r="C95" t="s">
-        <v>161</v>
+        <v>82</v>
       </c>
       <c r="D95" t="s">
-        <v>163</v>
+        <v>84</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B96" t="s">
-        <v>125</v>
+        <v>160</v>
       </c>
       <c r="C96" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="D96" t="s">
-        <v>125</v>
+        <v>162</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="B97" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="C97" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="D97" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B98" t="s">
-        <v>166</v>
+        <v>125</v>
       </c>
       <c r="C98" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="D98" t="s">
-        <v>166</v>
+        <v>125</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B99" t="s">
         <v>166</v>
       </c>
       <c r="C99" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D99" t="s">
         <v>166</v>
@@ -2375,69 +2408,69 @@
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="B100" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="C100" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D100" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="B101" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="C101" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D101" t="s">
-        <v>153</v>
+        <v>166</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="B102" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C102" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="D102" t="s">
-        <v>45</v>
+        <v>174</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B103" t="s">
-        <v>45</v>
+        <v>154</v>
       </c>
       <c r="C103" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="D103" t="s">
-        <v>45</v>
+        <v>153</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B104" t="s">
-        <v>45</v>
+        <v>176</v>
       </c>
       <c r="C104" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="D104" t="s">
         <v>45</v>
@@ -2445,13 +2478,13 @@
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B105" t="s">
         <v>45</v>
       </c>
       <c r="C105" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D105" t="s">
         <v>45</v>
@@ -2465,15 +2498,197 @@
         <v>45</v>
       </c>
       <c r="C106" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="D106" t="s">
         <v>45</v>
       </c>
     </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A107" t="s">
+        <v>181</v>
+      </c>
+      <c r="B107" t="s">
+        <v>45</v>
+      </c>
+      <c r="C107" t="s">
+        <v>182</v>
+      </c>
+      <c r="D107" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A108" t="s">
+        <v>181</v>
+      </c>
+      <c r="B108" t="s">
+        <v>45</v>
+      </c>
+      <c r="C108" t="s">
+        <v>183</v>
+      </c>
+      <c r="D108" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A109" t="s">
+        <v>181</v>
+      </c>
+      <c r="B109" t="s">
+        <v>45</v>
+      </c>
+      <c r="C109" t="s">
+        <v>181</v>
+      </c>
+      <c r="D109" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A110" t="s">
+        <v>181</v>
+      </c>
+      <c r="B110" t="s">
+        <v>45</v>
+      </c>
+      <c r="C110" t="s">
+        <v>186</v>
+      </c>
+      <c r="D110" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A111" t="s">
+        <v>164</v>
+      </c>
+      <c r="B111" t="s">
+        <v>125</v>
+      </c>
+      <c r="C111" t="s">
+        <v>165</v>
+      </c>
+      <c r="D111" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A112" t="s">
+        <v>181</v>
+      </c>
+      <c r="B112" t="s">
+        <v>45</v>
+      </c>
+      <c r="C112" t="s">
+        <v>184</v>
+      </c>
+      <c r="D112" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A113" t="s">
+        <v>185</v>
+      </c>
+      <c r="B113" t="s">
+        <v>142</v>
+      </c>
+      <c r="C113" t="s">
+        <v>185</v>
+      </c>
+      <c r="D113" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A114" t="s">
+        <v>51</v>
+      </c>
+      <c r="B114" t="s">
+        <v>52</v>
+      </c>
+      <c r="C114" t="s">
+        <v>188</v>
+      </c>
+      <c r="D114" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A115" t="s">
+        <v>135</v>
+      </c>
+      <c r="B115" t="s">
+        <v>56</v>
+      </c>
+      <c r="C115" t="s">
+        <v>189</v>
+      </c>
+      <c r="D115" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A116" t="s">
+        <v>135</v>
+      </c>
+      <c r="B116" t="s">
+        <v>56</v>
+      </c>
+      <c r="C116" t="s">
+        <v>134</v>
+      </c>
+      <c r="D116" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A117" t="s">
+        <v>190</v>
+      </c>
+      <c r="B117" t="s">
+        <v>141</v>
+      </c>
+      <c r="C117" t="s">
+        <v>190</v>
+      </c>
+      <c r="D117" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A118" t="s">
+        <v>192</v>
+      </c>
+      <c r="B118" t="s">
+        <v>194</v>
+      </c>
+      <c r="C118" t="s">
+        <v>191</v>
+      </c>
+      <c r="D118" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A119" t="s">
+        <v>192</v>
+      </c>
+      <c r="B119" t="s">
+        <v>194</v>
+      </c>
+      <c r="C119" t="s">
+        <v>193</v>
+      </c>
+      <c r="D119" t="s">
+        <v>194</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D93">
-    <sortCondition ref="A2:A93"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D95">
+    <sortCondition ref="A2:A95"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
15 module assembly coded this morning
</commit_message>
<xml_diff>
--- a/src/inputs/canonical_nodes.xlsx
+++ b/src/inputs/canonical_nodes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ben/Documents/bruegel/data_new/WORKING/INDUSTRY/tuone_v6/src/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC66DA15-3975-9344-B602-2A8F86A450A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C9B1087-7AD9-E24E-A92E-4E4231E9C660}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="720" windowWidth="29400" windowHeight="16940" xr2:uid="{EBC50A8D-91C7-594D-A950-AF99F2B3F4AF}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="198">
   <si>
     <t>Pylon LifeEU</t>
   </si>
@@ -622,6 +622,15 @@
   </si>
   <si>
     <t>Mercedes-Benz</t>
+  </si>
+  <si>
+    <t>Berlin-Marienfelde</t>
+  </si>
+  <si>
+    <t>Microvast</t>
+  </si>
+  <si>
+    <t>Ludwigsfelde</t>
   </si>
 </sst>
 </file>
@@ -1009,7 +1018,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DF9B3CA-7DC7-BB45-882F-C1DDB5BD93A3}">
-  <dimension ref="A1:E119"/>
+  <dimension ref="A1:E121"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.5" bestFit="1" customWidth="1"/>
@@ -2684,6 +2693,34 @@
       </c>
       <c r="D119" t="s">
         <v>194</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A120" t="s">
+        <v>195</v>
+      </c>
+      <c r="B120" t="s">
+        <v>194</v>
+      </c>
+      <c r="C120" t="s">
+        <v>105</v>
+      </c>
+      <c r="D120" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A121" t="s">
+        <v>197</v>
+      </c>
+      <c r="B121" t="s">
+        <v>196</v>
+      </c>
+      <c r="C121" t="s">
+        <v>109</v>
+      </c>
+      <c r="D121" t="s">
+        <v>196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
further module assembly validation
</commit_message>
<xml_diff>
--- a/src/inputs/canonical_nodes.xlsx
+++ b/src/inputs/canonical_nodes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ben/Documents/bruegel/data_new/WORKING/INDUSTRY/tuone_v6/src/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C9B1087-7AD9-E24E-A92E-4E4231E9C660}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D22BBCE3-40E2-B043-9BF8-1133EE933571}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="720" windowWidth="29400" windowHeight="16940" xr2:uid="{EBC50A8D-91C7-594D-A950-AF99F2B3F4AF}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="204">
   <si>
     <t>Pylon LifeEU</t>
   </si>
@@ -631,13 +631,31 @@
   </si>
   <si>
     <t>Ludwigsfelde</t>
+  </si>
+  <si>
+    <t>Impact Clean Power Technology</t>
+  </si>
+  <si>
+    <t>Warsaw</t>
+  </si>
+  <si>
+    <t>GigafactoryX</t>
+  </si>
+  <si>
+    <t>Pruszkow</t>
+  </si>
+  <si>
+    <t>Unipart Manufacturing Group</t>
+  </si>
+  <si>
+    <t>Hyperbat</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -657,6 +675,13 @@
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -680,10 +705,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1018,11 +1044,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DF9B3CA-7DC7-BB45-882F-C1DDB5BD93A3}">
-  <dimension ref="A1:E121"/>
+  <dimension ref="A1:E124"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.1640625" customWidth="1"/>
+    <col min="2" max="2" width="27.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="36.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19.1640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
@@ -2721,6 +2747,48 @@
       </c>
       <c r="D121" t="s">
         <v>196</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A122" t="s">
+        <v>199</v>
+      </c>
+      <c r="B122" t="s">
+        <v>198</v>
+      </c>
+      <c r="C122" t="s">
+        <v>200</v>
+      </c>
+      <c r="D122" s="3" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A123" t="s">
+        <v>199</v>
+      </c>
+      <c r="B123" t="s">
+        <v>198</v>
+      </c>
+      <c r="C123" t="s">
+        <v>201</v>
+      </c>
+      <c r="D123" s="3" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A124" t="s">
+        <v>98</v>
+      </c>
+      <c r="B124" t="s">
+        <v>203</v>
+      </c>
+      <c r="C124" t="s">
+        <v>98</v>
+      </c>
+      <c r="D124" t="s">
+        <v>202</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
finished validating battery cell projects for this version
</commit_message>
<xml_diff>
--- a/src/inputs/canonical_nodes.xlsx
+++ b/src/inputs/canonical_nodes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ben/Documents/bruegel/data_new/WORKING/INDUSTRY/tuone_v6/src/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D22BBCE3-40E2-B043-9BF8-1133EE933571}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40F836FF-0DD0-F945-B4DB-D92E46CAEDFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="720" windowWidth="29400" windowHeight="16940" xr2:uid="{EBC50A8D-91C7-594D-A950-AF99F2B3F4AF}"/>
+    <workbookView xWindow="0" yWindow="820" windowWidth="29400" windowHeight="16940" xr2:uid="{EBC50A8D-91C7-594D-A950-AF99F2B3F4AF}"/>
   </bookViews>
   <sheets>
     <sheet name="merge" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="211">
   <si>
     <t>Pylon LifeEU</t>
   </si>
@@ -649,6 +649,27 @@
   </si>
   <si>
     <t>Hyperbat</t>
+  </si>
+  <si>
+    <t>Rimac Automobilii</t>
+  </si>
+  <si>
+    <t>Zagreb</t>
+  </si>
+  <si>
+    <t>Rimac Automobili</t>
+  </si>
+  <si>
+    <t>Scania</t>
+  </si>
+  <si>
+    <t>Västerås</t>
+  </si>
+  <si>
+    <t>Stuttgart</t>
+  </si>
+  <si>
+    <t>Stuttgart-Untertürkheim</t>
   </si>
 </sst>
 </file>
@@ -1044,7 +1065,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DF9B3CA-7DC7-BB45-882F-C1DDB5BD93A3}">
-  <dimension ref="A1:E124"/>
+  <dimension ref="A1:E130"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.5" bestFit="1" customWidth="1"/>
@@ -1113,44 +1134,44 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>76</v>
+        <v>168</v>
       </c>
       <c r="B5" t="s">
-        <v>75</v>
+        <v>166</v>
       </c>
       <c r="C5" t="s">
-        <v>76</v>
+        <v>171</v>
       </c>
       <c r="D5" t="s">
-        <v>77</v>
+        <v>166</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>113</v>
+        <v>76</v>
       </c>
       <c r="B6" t="s">
-        <v>114</v>
+        <v>75</v>
       </c>
       <c r="C6" t="s">
-        <v>115</v>
+        <v>76</v>
       </c>
       <c r="D6" t="s">
-        <v>114</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>113</v>
+        <v>195</v>
       </c>
       <c r="B7" t="s">
-        <v>114</v>
+        <v>194</v>
       </c>
       <c r="C7" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="D7" t="s">
-        <v>114</v>
+        <v>194</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -1158,83 +1179,83 @@
         <v>113</v>
       </c>
       <c r="B8" t="s">
-        <v>158</v>
+        <v>114</v>
       </c>
       <c r="C8" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D8" t="s">
-        <v>158</v>
+        <v>114</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="B9" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="C9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D9" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="B10" t="s">
-        <v>119</v>
+        <v>158</v>
       </c>
       <c r="C10" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D10" t="s">
-        <v>119</v>
+        <v>158</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>85</v>
+        <v>118</v>
       </c>
       <c r="B11" t="s">
-        <v>86</v>
+        <v>119</v>
       </c>
       <c r="C11" t="s">
-        <v>85</v>
+        <v>117</v>
       </c>
       <c r="D11" t="s">
-        <v>87</v>
+        <v>119</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>30</v>
+        <v>118</v>
       </c>
       <c r="B12" t="s">
-        <v>31</v>
+        <v>119</v>
       </c>
       <c r="C12" t="s">
-        <v>32</v>
+        <v>120</v>
       </c>
       <c r="D12" t="s">
-        <v>31</v>
+        <v>119</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>30</v>
+        <v>85</v>
       </c>
       <c r="B13" t="s">
-        <v>31</v>
+        <v>86</v>
       </c>
       <c r="C13" t="s">
-        <v>32</v>
+        <v>85</v>
       </c>
       <c r="D13" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
@@ -1245,10 +1266,10 @@
         <v>31</v>
       </c>
       <c r="C14" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D14" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
@@ -1259,10 +1280,10 @@
         <v>31</v>
       </c>
       <c r="C15" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D15" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
@@ -1276,959 +1297,959 @@
         <v>30</v>
       </c>
       <c r="D16" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>128</v>
+        <v>30</v>
       </c>
       <c r="B17" t="s">
-        <v>130</v>
+        <v>31</v>
       </c>
       <c r="C17" t="s">
-        <v>129</v>
+        <v>30</v>
       </c>
       <c r="D17" t="s">
-        <v>130</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>98</v>
+        <v>30</v>
       </c>
       <c r="B18" t="s">
-        <v>99</v>
+        <v>31</v>
       </c>
       <c r="C18" t="s">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="D18" t="s">
-        <v>99</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>146</v>
+        <v>128</v>
       </c>
       <c r="B19" t="s">
-        <v>147</v>
+        <v>130</v>
       </c>
       <c r="C19" t="s">
-        <v>148</v>
+        <v>129</v>
       </c>
       <c r="D19" t="s">
-        <v>147</v>
+        <v>130</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>146</v>
+        <v>98</v>
       </c>
       <c r="B20" t="s">
-        <v>147</v>
+        <v>99</v>
       </c>
       <c r="C20" t="s">
-        <v>149</v>
+        <v>100</v>
       </c>
       <c r="D20" t="s">
-        <v>147</v>
+        <v>99</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>134</v>
+        <v>98</v>
       </c>
       <c r="B21" t="s">
-        <v>56</v>
+        <v>203</v>
       </c>
       <c r="C21" t="s">
-        <v>135</v>
+        <v>98</v>
       </c>
       <c r="D21" t="s">
-        <v>56</v>
+        <v>202</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="B22" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C22" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="D22" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="B23" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C23" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D23" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>152</v>
+        <v>134</v>
       </c>
       <c r="B24" t="s">
-        <v>151</v>
+        <v>56</v>
       </c>
       <c r="C24" t="s">
-        <v>152</v>
+        <v>135</v>
       </c>
       <c r="D24" t="s">
-        <v>155</v>
+        <v>56</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="B25" t="s">
-        <v>25</v>
+        <v>56</v>
       </c>
       <c r="C25" t="s">
-        <v>121</v>
+        <v>189</v>
       </c>
       <c r="D25" t="s">
-        <v>20</v>
+        <v>56</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>157</v>
+        <v>134</v>
       </c>
       <c r="B26" t="s">
-        <v>156</v>
+        <v>56</v>
       </c>
       <c r="C26" t="s">
-        <v>152</v>
+        <v>135</v>
       </c>
       <c r="D26" t="s">
-        <v>156</v>
+        <v>56</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>101</v>
+        <v>152</v>
       </c>
       <c r="B27" t="s">
-        <v>84</v>
+        <v>151</v>
       </c>
       <c r="C27" t="s">
-        <v>102</v>
+        <v>152</v>
       </c>
       <c r="D27" t="s">
-        <v>84</v>
+        <v>153</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>101</v>
+        <v>152</v>
       </c>
       <c r="B28" t="s">
-        <v>84</v>
+        <v>151</v>
       </c>
       <c r="C28" t="s">
-        <v>103</v>
+        <v>152</v>
       </c>
       <c r="D28" t="s">
-        <v>84</v>
+        <v>154</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>101</v>
+        <v>152</v>
       </c>
       <c r="B29" t="s">
-        <v>84</v>
+        <v>151</v>
       </c>
       <c r="C29" t="s">
-        <v>104</v>
+        <v>152</v>
       </c>
       <c r="D29" t="s">
-        <v>84</v>
+        <v>155</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="B30" t="s">
-        <v>125</v>
+        <v>25</v>
       </c>
       <c r="C30" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="D30" t="s">
-        <v>125</v>
+        <v>20</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>67</v>
+        <v>157</v>
       </c>
       <c r="B31" t="s">
-        <v>66</v>
+        <v>156</v>
       </c>
       <c r="C31" t="s">
-        <v>67</v>
+        <v>152</v>
       </c>
       <c r="D31" t="s">
-        <v>68</v>
+        <v>156</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>70</v>
+        <v>101</v>
       </c>
       <c r="B32" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="C32" t="s">
-        <v>70</v>
+        <v>102</v>
       </c>
       <c r="D32" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>70</v>
+        <v>101</v>
       </c>
       <c r="B33" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="C33" t="s">
-        <v>70</v>
+        <v>103</v>
       </c>
       <c r="D33" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>70</v>
+        <v>101</v>
       </c>
       <c r="B34" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="C34" t="s">
-        <v>70</v>
+        <v>104</v>
       </c>
       <c r="D34" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>107</v>
+        <v>127</v>
       </c>
       <c r="B35" t="s">
-        <v>69</v>
+        <v>125</v>
       </c>
       <c r="C35" t="s">
-        <v>106</v>
+        <v>126</v>
       </c>
       <c r="D35" t="s">
-        <v>69</v>
+        <v>125</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>107</v>
+        <v>67</v>
       </c>
       <c r="B36" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C36" t="s">
-        <v>105</v>
+        <v>67</v>
       </c>
       <c r="D36" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>107</v>
+        <v>164</v>
       </c>
       <c r="B37" t="s">
-        <v>69</v>
+        <v>125</v>
       </c>
       <c r="C37" t="s">
-        <v>108</v>
+        <v>165</v>
       </c>
       <c r="D37" t="s">
-        <v>69</v>
+        <v>125</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>107</v>
+        <v>164</v>
       </c>
       <c r="B38" t="s">
-        <v>69</v>
+        <v>125</v>
       </c>
       <c r="C38" t="s">
-        <v>109</v>
+        <v>165</v>
       </c>
       <c r="D38" t="s">
-        <v>69</v>
+        <v>125</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>107</v>
+        <v>70</v>
       </c>
       <c r="B39" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C39" t="s">
-        <v>110</v>
+        <v>70</v>
       </c>
       <c r="D39" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>107</v>
+        <v>70</v>
       </c>
       <c r="B40" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C40" t="s">
-        <v>111</v>
+        <v>70</v>
       </c>
       <c r="D40" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>107</v>
+        <v>70</v>
       </c>
       <c r="B41" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C41" t="s">
-        <v>112</v>
+        <v>70</v>
       </c>
       <c r="D41" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>139</v>
+        <v>107</v>
       </c>
       <c r="B42" t="s">
-        <v>25</v>
+        <v>69</v>
       </c>
       <c r="C42" t="s">
-        <v>139</v>
+        <v>106</v>
       </c>
       <c r="D42" t="s">
-        <v>140</v>
+        <v>69</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>139</v>
+        <v>107</v>
       </c>
       <c r="B43" t="s">
-        <v>25</v>
+        <v>69</v>
       </c>
       <c r="C43" t="s">
-        <v>139</v>
+        <v>105</v>
       </c>
       <c r="D43" t="s">
-        <v>141</v>
+        <v>69</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>139</v>
+        <v>107</v>
       </c>
       <c r="B44" t="s">
-        <v>25</v>
+        <v>69</v>
       </c>
       <c r="C44" t="s">
-        <v>139</v>
+        <v>108</v>
       </c>
       <c r="D44" t="s">
-        <v>142</v>
+        <v>69</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>139</v>
+        <v>107</v>
       </c>
       <c r="B45" t="s">
-        <v>25</v>
+        <v>69</v>
       </c>
       <c r="C45" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="D45" t="s">
-        <v>20</v>
+        <v>69</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>131</v>
+        <v>107</v>
       </c>
       <c r="B46" t="s">
-        <v>132</v>
+        <v>69</v>
       </c>
       <c r="C46" t="s">
-        <v>133</v>
+        <v>110</v>
       </c>
       <c r="D46" t="s">
-        <v>132</v>
+        <v>69</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>5</v>
+        <v>107</v>
       </c>
       <c r="B47" t="s">
-        <v>6</v>
+        <v>69</v>
       </c>
       <c r="C47" t="s">
-        <v>5</v>
+        <v>111</v>
       </c>
       <c r="D47" t="s">
-        <v>7</v>
+        <v>69</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>78</v>
+        <v>107</v>
       </c>
       <c r="B48" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="C48" t="s">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="D48" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>78</v>
+        <v>177</v>
       </c>
       <c r="B49" t="s">
-        <v>79</v>
+        <v>176</v>
       </c>
       <c r="C49" t="s">
-        <v>78</v>
+        <v>177</v>
       </c>
       <c r="D49" t="s">
-        <v>81</v>
+        <v>45</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>62</v>
+        <v>178</v>
       </c>
       <c r="B50" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="C50" t="s">
-        <v>62</v>
+        <v>179</v>
       </c>
       <c r="D50" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>62</v>
+        <v>139</v>
       </c>
       <c r="B51" t="s">
-        <v>61</v>
+        <v>25</v>
       </c>
       <c r="C51" t="s">
-        <v>62</v>
+        <v>139</v>
       </c>
       <c r="D51" t="s">
-        <v>52</v>
+        <v>140</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>21</v>
+        <v>139</v>
       </c>
       <c r="B52" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C52" t="s">
-        <v>21</v>
+        <v>139</v>
       </c>
       <c r="D52" t="s">
-        <v>22</v>
+        <v>141</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>21</v>
+        <v>139</v>
       </c>
       <c r="B53" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C53" t="s">
-        <v>21</v>
+        <v>139</v>
       </c>
       <c r="D53" t="s">
-        <v>23</v>
+        <v>142</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>21</v>
+        <v>139</v>
       </c>
       <c r="B54" t="s">
+        <v>25</v>
+      </c>
+      <c r="C54" t="s">
+        <v>139</v>
+      </c>
+      <c r="D54" t="s">
         <v>20</v>
-      </c>
-      <c r="C54" t="s">
-        <v>38</v>
-      </c>
-      <c r="D54" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>21</v>
+        <v>167</v>
       </c>
       <c r="B55" t="s">
-        <v>20</v>
+        <v>166</v>
       </c>
       <c r="C55" t="s">
-        <v>24</v>
+        <v>169</v>
       </c>
       <c r="D55" t="s">
-        <v>22</v>
+        <v>166</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>21</v>
+        <v>167</v>
       </c>
       <c r="B56" t="s">
-        <v>20</v>
+        <v>166</v>
       </c>
       <c r="C56" t="s">
-        <v>24</v>
+        <v>170</v>
       </c>
       <c r="D56" t="s">
-        <v>23</v>
+        <v>166</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>21</v>
+        <v>131</v>
       </c>
       <c r="B57" t="s">
-        <v>20</v>
+        <v>132</v>
       </c>
       <c r="C57" t="s">
-        <v>24</v>
+        <v>133</v>
       </c>
       <c r="D57" t="s">
-        <v>20</v>
+        <v>132</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="B58" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="C58" t="s">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="D58" t="s">
-        <v>40</v>
+        <v>7</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>144</v>
+        <v>197</v>
       </c>
       <c r="B59" t="s">
-        <v>143</v>
+        <v>196</v>
       </c>
       <c r="C59" t="s">
-        <v>145</v>
+        <v>109</v>
       </c>
       <c r="D59" t="s">
-        <v>143</v>
+        <v>196</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="B60" t="s">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="C60" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="D60" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="B61" t="s">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="C61" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="D61" t="s">
-        <v>64</v>
+        <v>81</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B62" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="C62" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="D62" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B63" t="s">
+        <v>61</v>
+      </c>
+      <c r="C63" t="s">
+        <v>62</v>
+      </c>
+      <c r="D63" t="s">
         <v>52</v>
-      </c>
-      <c r="C63" t="s">
-        <v>59</v>
-      </c>
-      <c r="D63" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>59</v>
+        <v>21</v>
       </c>
       <c r="B64" t="s">
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="C64" t="s">
-        <v>59</v>
+        <v>21</v>
       </c>
       <c r="D64" t="s">
-        <v>60</v>
+        <v>22</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="B65" t="s">
         <v>20</v>
       </c>
       <c r="C65" t="s">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="D65" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="B66" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="C66" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="D66" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="B67" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="C67" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="D67" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="B68" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="C68" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="D68" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="B69" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="C69" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D69" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>51</v>
+        <v>21</v>
       </c>
       <c r="B70" t="s">
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="C70" t="s">
-        <v>53</v>
+        <v>24</v>
       </c>
       <c r="D70" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>54</v>
+        <v>144</v>
       </c>
       <c r="B71" t="s">
-        <v>55</v>
+        <v>143</v>
       </c>
       <c r="C71" t="s">
-        <v>54</v>
+        <v>145</v>
       </c>
       <c r="D71" t="s">
-        <v>56</v>
+        <v>143</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>3</v>
+        <v>63</v>
       </c>
       <c r="B72" t="s">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="C72" t="s">
-        <v>1</v>
+        <v>65</v>
       </c>
       <c r="D72" t="s">
-        <v>2</v>
+        <v>64</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>3</v>
+        <v>63</v>
       </c>
       <c r="B73" t="s">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="C73" t="s">
-        <v>1</v>
+        <v>65</v>
       </c>
       <c r="D73" t="s">
-        <v>4</v>
+        <v>64</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>3</v>
+        <v>175</v>
       </c>
       <c r="B74" t="s">
-        <v>0</v>
+        <v>154</v>
       </c>
       <c r="C74" t="s">
-        <v>3</v>
+        <v>175</v>
       </c>
       <c r="D74" t="s">
-        <v>2</v>
+        <v>153</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>3</v>
+        <v>57</v>
       </c>
       <c r="B75" t="s">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="C75" t="s">
-        <v>3</v>
+        <v>57</v>
       </c>
       <c r="D75" t="s">
-        <v>4</v>
+        <v>58</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>89</v>
+        <v>185</v>
       </c>
       <c r="B76" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="C76" t="s">
-        <v>89</v>
+        <v>185</v>
       </c>
       <c r="D76" t="s">
-        <v>88</v>
+        <v>20</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>89</v>
+        <v>59</v>
       </c>
       <c r="B77" t="s">
-        <v>90</v>
+        <v>52</v>
       </c>
       <c r="C77" t="s">
-        <v>89</v>
+        <v>59</v>
       </c>
       <c r="D77" t="s">
-        <v>91</v>
+        <v>58</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>8</v>
+        <v>59</v>
       </c>
       <c r="B78" t="s">
-        <v>10</v>
+        <v>52</v>
       </c>
       <c r="C78" t="s">
-        <v>9</v>
+        <v>59</v>
       </c>
       <c r="D78" t="s">
-        <v>10</v>
+        <v>60</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>44</v>
+        <v>173</v>
       </c>
       <c r="B79" t="s">
-        <v>43</v>
+        <v>174</v>
       </c>
       <c r="C79" t="s">
-        <v>44</v>
+        <v>172</v>
       </c>
       <c r="D79" t="s">
-        <v>45</v>
+        <v>174</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>159</v>
+        <v>39</v>
       </c>
       <c r="B80" t="s">
-        <v>151</v>
+        <v>20</v>
       </c>
       <c r="C80" t="s">
-        <v>159</v>
+        <v>39</v>
       </c>
       <c r="D80" t="s">
-        <v>154</v>
+        <v>22</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>159</v>
+        <v>12</v>
       </c>
       <c r="B81" t="s">
-        <v>151</v>
+        <v>11</v>
       </c>
       <c r="C81" t="s">
-        <v>159</v>
+        <v>12</v>
       </c>
       <c r="D81" t="s">
-        <v>153</v>
+        <v>13</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>92</v>
+        <v>12</v>
       </c>
       <c r="B82" t="s">
-        <v>79</v>
+        <v>11</v>
       </c>
       <c r="C82" t="s">
-        <v>92</v>
+        <v>12</v>
       </c>
       <c r="D82" t="s">
-        <v>81</v>
+        <v>14</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>92</v>
+        <v>12</v>
       </c>
       <c r="B83" t="s">
-        <v>79</v>
+        <v>11</v>
       </c>
       <c r="C83" t="s">
-        <v>92</v>
+        <v>15</v>
       </c>
       <c r="D83" t="s">
-        <v>80</v>
+        <v>14</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>26</v>
+        <v>187</v>
       </c>
       <c r="B84" t="s">
-        <v>25</v>
+        <v>74</v>
       </c>
       <c r="C84" t="s">
-        <v>20</v>
+        <v>137</v>
       </c>
       <c r="D84" t="s">
-        <v>26</v>
+        <v>138</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.2">
@@ -2242,7 +2263,7 @@
         <v>137</v>
       </c>
       <c r="D85" t="s">
-        <v>138</v>
+        <v>74</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.2">
@@ -2253,10 +2274,10 @@
         <v>74</v>
       </c>
       <c r="C86" t="s">
-        <v>137</v>
+        <v>150</v>
       </c>
       <c r="D86" t="s">
-        <v>74</v>
+        <v>138</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.2">
@@ -2267,10 +2288,10 @@
         <v>74</v>
       </c>
       <c r="C87" t="s">
-        <v>150</v>
+        <v>137</v>
       </c>
       <c r="D87" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.2">
@@ -2281,245 +2302,245 @@
         <v>74</v>
       </c>
       <c r="C88" t="s">
-        <v>137</v>
+        <v>187</v>
       </c>
       <c r="D88" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="B89" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="C89" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="D89" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>96</v>
+        <v>51</v>
       </c>
       <c r="B90" t="s">
-        <v>95</v>
+        <v>52</v>
       </c>
       <c r="C90" t="s">
-        <v>97</v>
+        <v>53</v>
       </c>
       <c r="D90" t="s">
-        <v>95</v>
+        <v>52</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B91" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="C91" t="s">
-        <v>48</v>
+        <v>188</v>
       </c>
       <c r="D91" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="B92" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="C92" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D92" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>46</v>
+        <v>3</v>
       </c>
       <c r="B93" t="s">
-        <v>47</v>
+        <v>0</v>
       </c>
       <c r="C93" t="s">
-        <v>49</v>
+        <v>1</v>
       </c>
       <c r="D93" t="s">
-        <v>50</v>
+        <v>2</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>82</v>
+        <v>3</v>
       </c>
       <c r="B94" t="s">
-        <v>83</v>
+        <v>0</v>
       </c>
       <c r="C94" t="s">
-        <v>82</v>
+        <v>1</v>
       </c>
       <c r="D94" t="s">
-        <v>20</v>
+        <v>4</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>82</v>
+        <v>3</v>
       </c>
       <c r="B95" t="s">
-        <v>83</v>
+        <v>0</v>
       </c>
       <c r="C95" t="s">
-        <v>82</v>
+        <v>3</v>
       </c>
       <c r="D95" t="s">
-        <v>84</v>
+        <v>2</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>161</v>
+        <v>3</v>
       </c>
       <c r="B96" t="s">
-        <v>160</v>
+        <v>0</v>
       </c>
       <c r="C96" t="s">
-        <v>161</v>
+        <v>3</v>
       </c>
       <c r="D96" t="s">
-        <v>162</v>
+        <v>4</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>161</v>
+        <v>89</v>
       </c>
       <c r="B97" t="s">
-        <v>160</v>
+        <v>90</v>
       </c>
       <c r="C97" t="s">
-        <v>161</v>
+        <v>89</v>
       </c>
       <c r="D97" t="s">
-        <v>163</v>
+        <v>88</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>164</v>
+        <v>89</v>
       </c>
       <c r="B98" t="s">
-        <v>125</v>
+        <v>90</v>
       </c>
       <c r="C98" t="s">
-        <v>165</v>
+        <v>89</v>
       </c>
       <c r="D98" t="s">
-        <v>125</v>
+        <v>91</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>167</v>
+        <v>8</v>
       </c>
       <c r="B99" t="s">
-        <v>166</v>
+        <v>10</v>
       </c>
       <c r="C99" t="s">
-        <v>169</v>
+        <v>9</v>
       </c>
       <c r="D99" t="s">
-        <v>166</v>
+        <v>10</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>167</v>
+        <v>44</v>
       </c>
       <c r="B100" t="s">
-        <v>166</v>
+        <v>43</v>
       </c>
       <c r="C100" t="s">
-        <v>170</v>
+        <v>44</v>
       </c>
       <c r="D100" t="s">
-        <v>166</v>
+        <v>45</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>168</v>
+        <v>181</v>
       </c>
       <c r="B101" t="s">
-        <v>166</v>
+        <v>45</v>
       </c>
       <c r="C101" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="D101" t="s">
-        <v>166</v>
+        <v>45</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="B102" t="s">
-        <v>174</v>
+        <v>45</v>
       </c>
       <c r="C102" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
       <c r="D102" t="s">
-        <v>174</v>
+        <v>45</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="B103" t="s">
-        <v>154</v>
+        <v>45</v>
       </c>
       <c r="C103" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="D103" t="s">
-        <v>153</v>
+        <v>45</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="B104" t="s">
-        <v>176</v>
+        <v>45</v>
       </c>
       <c r="C104" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="D104" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B105" t="s">
         <v>45</v>
       </c>
       <c r="C105" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="D105" t="s">
         <v>45</v>
@@ -2533,7 +2554,7 @@
         <v>45</v>
       </c>
       <c r="C106" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="D106" t="s">
         <v>45</v>
@@ -2541,167 +2562,167 @@
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>181</v>
+        <v>159</v>
       </c>
       <c r="B107" t="s">
-        <v>45</v>
+        <v>151</v>
       </c>
       <c r="C107" t="s">
-        <v>182</v>
+        <v>159</v>
       </c>
       <c r="D107" t="s">
-        <v>45</v>
+        <v>154</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>181</v>
+        <v>159</v>
       </c>
       <c r="B108" t="s">
-        <v>45</v>
+        <v>151</v>
       </c>
       <c r="C108" t="s">
-        <v>183</v>
+        <v>159</v>
       </c>
       <c r="D108" t="s">
-        <v>45</v>
+        <v>153</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="B109" t="s">
-        <v>45</v>
+        <v>160</v>
       </c>
       <c r="C109" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D109" t="s">
-        <v>52</v>
+        <v>162</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="B110" t="s">
-        <v>45</v>
+        <v>160</v>
       </c>
       <c r="C110" t="s">
-        <v>186</v>
+        <v>161</v>
       </c>
       <c r="D110" t="s">
-        <v>45</v>
+        <v>163</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
-        <v>164</v>
+        <v>92</v>
       </c>
       <c r="B111" t="s">
-        <v>125</v>
+        <v>79</v>
       </c>
       <c r="C111" t="s">
-        <v>165</v>
+        <v>92</v>
       </c>
       <c r="D111" t="s">
-        <v>125</v>
+        <v>81</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>181</v>
+        <v>92</v>
       </c>
       <c r="B112" t="s">
-        <v>45</v>
+        <v>79</v>
       </c>
       <c r="C112" t="s">
-        <v>184</v>
+        <v>92</v>
       </c>
       <c r="D112" t="s">
-        <v>45</v>
+        <v>80</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
-        <v>185</v>
+        <v>26</v>
       </c>
       <c r="B113" t="s">
-        <v>142</v>
+        <v>25</v>
       </c>
       <c r="C113" t="s">
-        <v>185</v>
+        <v>20</v>
       </c>
       <c r="D113" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
-        <v>51</v>
+        <v>190</v>
       </c>
       <c r="B114" t="s">
-        <v>52</v>
+        <v>141</v>
       </c>
       <c r="C114" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D114" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
-        <v>135</v>
+        <v>24</v>
       </c>
       <c r="B115" t="s">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="C115" t="s">
-        <v>189</v>
+        <v>24</v>
       </c>
       <c r="D115" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
-        <v>135</v>
+        <v>209</v>
       </c>
       <c r="B116" t="s">
-        <v>56</v>
+        <v>194</v>
       </c>
       <c r="C116" t="s">
-        <v>134</v>
+        <v>191</v>
       </c>
       <c r="D116" t="s">
-        <v>56</v>
+        <v>194</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
-        <v>190</v>
+        <v>209</v>
       </c>
       <c r="B117" t="s">
-        <v>141</v>
+        <v>194</v>
       </c>
       <c r="C117" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="D117" t="s">
-        <v>40</v>
+        <v>194</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
-        <v>192</v>
+        <v>209</v>
       </c>
       <c r="B118" t="s">
         <v>194</v>
       </c>
       <c r="C118" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D118" t="s">
         <v>194</v>
@@ -2709,13 +2730,13 @@
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
-        <v>192</v>
+        <v>209</v>
       </c>
       <c r="B119" t="s">
         <v>194</v>
       </c>
       <c r="C119" t="s">
-        <v>193</v>
+        <v>210</v>
       </c>
       <c r="D119" t="s">
         <v>194</v>
@@ -2723,77 +2744,161 @@
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
-        <v>195</v>
+        <v>208</v>
       </c>
       <c r="B120" t="s">
-        <v>194</v>
+        <v>45</v>
       </c>
       <c r="C120" t="s">
-        <v>105</v>
+        <v>208</v>
       </c>
       <c r="D120" t="s">
-        <v>194</v>
+        <v>207</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
-        <v>197</v>
+        <v>96</v>
       </c>
       <c r="B121" t="s">
-        <v>196</v>
+        <v>95</v>
       </c>
       <c r="C121" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="D121" t="s">
-        <v>196</v>
+        <v>95</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
-        <v>199</v>
+        <v>46</v>
       </c>
       <c r="B122" t="s">
-        <v>198</v>
+        <v>47</v>
       </c>
       <c r="C122" t="s">
-        <v>200</v>
-      </c>
-      <c r="D122" s="3" t="s">
-        <v>198</v>
+        <v>48</v>
+      </c>
+      <c r="D122" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
-        <v>199</v>
+        <v>46</v>
       </c>
       <c r="B123" t="s">
-        <v>198</v>
+        <v>47</v>
       </c>
       <c r="C123" t="s">
-        <v>201</v>
-      </c>
-      <c r="D123" s="3" t="s">
-        <v>198</v>
+        <v>49</v>
+      </c>
+      <c r="D123" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
-        <v>98</v>
+        <v>46</v>
       </c>
       <c r="B124" t="s">
-        <v>203</v>
+        <v>47</v>
       </c>
       <c r="C124" t="s">
-        <v>98</v>
+        <v>49</v>
       </c>
       <c r="D124" t="s">
-        <v>202</v>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A125" t="s">
+        <v>199</v>
+      </c>
+      <c r="B125" t="s">
+        <v>198</v>
+      </c>
+      <c r="C125" t="s">
+        <v>200</v>
+      </c>
+      <c r="D125" s="3" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A126" t="s">
+        <v>199</v>
+      </c>
+      <c r="B126" t="s">
+        <v>198</v>
+      </c>
+      <c r="C126" t="s">
+        <v>201</v>
+      </c>
+      <c r="D126" s="3" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A127" t="s">
+        <v>205</v>
+      </c>
+      <c r="B127" t="s">
+        <v>206</v>
+      </c>
+      <c r="C127" t="s">
+        <v>205</v>
+      </c>
+      <c r="D127" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A128" t="s">
+        <v>82</v>
+      </c>
+      <c r="B128" t="s">
+        <v>83</v>
+      </c>
+      <c r="C128" t="s">
+        <v>82</v>
+      </c>
+      <c r="D128" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A129" t="s">
+        <v>82</v>
+      </c>
+      <c r="B129" t="s">
+        <v>83</v>
+      </c>
+      <c r="C129" t="s">
+        <v>82</v>
+      </c>
+      <c r="D129" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A130" t="s">
+        <v>109</v>
+      </c>
+      <c r="B130" t="s">
+        <v>74</v>
+      </c>
+      <c r="C130" t="s">
+        <v>109</v>
+      </c>
+      <c r="D130" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D95">
-    <sortCondition ref="A2:A95"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D129">
+    <sortCondition ref="A2:A129"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
another 20 module assembly validated
</commit_message>
<xml_diff>
--- a/src/inputs/canonical_nodes.xlsx
+++ b/src/inputs/canonical_nodes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ben/Documents/bruegel/data_new/WORKING/INDUSTRY/tuone_v6/src/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40F836FF-0DD0-F945-B4DB-D92E46CAEDFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38B2AC9C-C963-7C46-BDD7-73FF5F28249A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="820" windowWidth="29400" windowHeight="16940" xr2:uid="{EBC50A8D-91C7-594D-A950-AF99F2B3F4AF}"/>
+    <workbookView xWindow="0" yWindow="800" windowWidth="29400" windowHeight="16940" xr2:uid="{EBC50A8D-91C7-594D-A950-AF99F2B3F4AF}"/>
   </bookViews>
   <sheets>
     <sheet name="merge" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="208">
   <si>
     <t>Pylon LifeEU</t>
   </si>
@@ -612,9 +612,6 @@
     <t>Trnava</t>
   </si>
   <si>
-    <t>Untertürkheim Hedelfingen</t>
-  </si>
-  <si>
     <t>Untertürkheim</t>
   </si>
   <si>
@@ -664,12 +661,6 @@
   </si>
   <si>
     <t>Västerås</t>
-  </si>
-  <si>
-    <t>Stuttgart</t>
-  </si>
-  <si>
-    <t>Stuttgart-Untertürkheim</t>
   </si>
 </sst>
 </file>
@@ -1065,7 +1056,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DF9B3CA-7DC7-BB45-882F-C1DDB5BD93A3}">
-  <dimension ref="A1:E130"/>
+  <dimension ref="A1:E127"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.5" bestFit="1" customWidth="1"/>
@@ -1162,16 +1153,16 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B7" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C7" t="s">
         <v>105</v>
       </c>
       <c r="D7" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -1218,16 +1209,16 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="B11" t="s">
-        <v>119</v>
+        <v>74</v>
       </c>
       <c r="C11" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="D11" t="s">
-        <v>119</v>
+        <v>138</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
@@ -1238,7 +1229,7 @@
         <v>119</v>
       </c>
       <c r="C12" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="D12" t="s">
         <v>119</v>
@@ -1246,30 +1237,30 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>85</v>
+        <v>118</v>
       </c>
       <c r="B13" t="s">
-        <v>86</v>
+        <v>119</v>
       </c>
       <c r="C13" t="s">
-        <v>85</v>
+        <v>120</v>
       </c>
       <c r="D13" t="s">
-        <v>87</v>
+        <v>119</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>30</v>
+        <v>85</v>
       </c>
       <c r="B14" t="s">
-        <v>31</v>
+        <v>86</v>
       </c>
       <c r="C14" t="s">
-        <v>32</v>
+        <v>85</v>
       </c>
       <c r="D14" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
@@ -1294,10 +1285,10 @@
         <v>31</v>
       </c>
       <c r="C16" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D16" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
@@ -1311,7 +1302,7 @@
         <v>30</v>
       </c>
       <c r="D17" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
@@ -1325,35 +1316,35 @@
         <v>30</v>
       </c>
       <c r="D18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>128</v>
+        <v>30</v>
       </c>
       <c r="B19" t="s">
-        <v>130</v>
+        <v>31</v>
       </c>
       <c r="C19" t="s">
-        <v>129</v>
+        <v>30</v>
       </c>
       <c r="D19" t="s">
-        <v>130</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>98</v>
+        <v>128</v>
       </c>
       <c r="B20" t="s">
-        <v>99</v>
+        <v>130</v>
       </c>
       <c r="C20" t="s">
-        <v>100</v>
+        <v>129</v>
       </c>
       <c r="D20" t="s">
-        <v>99</v>
+        <v>130</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
@@ -1361,27 +1352,27 @@
         <v>98</v>
       </c>
       <c r="B21" t="s">
-        <v>203</v>
+        <v>99</v>
       </c>
       <c r="C21" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D21" t="s">
-        <v>202</v>
+        <v>99</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>146</v>
+        <v>98</v>
       </c>
       <c r="B22" t="s">
-        <v>147</v>
+        <v>202</v>
       </c>
       <c r="C22" t="s">
-        <v>148</v>
+        <v>98</v>
       </c>
       <c r="D22" t="s">
-        <v>147</v>
+        <v>201</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
@@ -1392,7 +1383,7 @@
         <v>147</v>
       </c>
       <c r="C23" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D23" t="s">
         <v>147</v>
@@ -1400,16 +1391,16 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
       <c r="B24" t="s">
-        <v>56</v>
+        <v>147</v>
       </c>
       <c r="C24" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="D24" t="s">
-        <v>56</v>
+        <v>147</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
@@ -1420,7 +1411,7 @@
         <v>56</v>
       </c>
       <c r="C25" t="s">
-        <v>189</v>
+        <v>135</v>
       </c>
       <c r="D25" t="s">
         <v>56</v>
@@ -1434,7 +1425,7 @@
         <v>56</v>
       </c>
       <c r="C26" t="s">
-        <v>135</v>
+        <v>189</v>
       </c>
       <c r="D26" t="s">
         <v>56</v>
@@ -1442,16 +1433,16 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>152</v>
+        <v>134</v>
       </c>
       <c r="B27" t="s">
-        <v>151</v>
+        <v>56</v>
       </c>
       <c r="C27" t="s">
-        <v>152</v>
+        <v>135</v>
       </c>
       <c r="D27" t="s">
-        <v>153</v>
+        <v>56</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
@@ -1465,7 +1456,7 @@
         <v>152</v>
       </c>
       <c r="D28" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
@@ -1479,49 +1470,49 @@
         <v>152</v>
       </c>
       <c r="D29" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>121</v>
+        <v>152</v>
       </c>
       <c r="B30" t="s">
-        <v>25</v>
+        <v>151</v>
       </c>
       <c r="C30" t="s">
-        <v>121</v>
+        <v>152</v>
       </c>
       <c r="D30" t="s">
-        <v>20</v>
+        <v>155</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>157</v>
+        <v>121</v>
       </c>
       <c r="B31" t="s">
-        <v>156</v>
+        <v>25</v>
       </c>
       <c r="C31" t="s">
-        <v>152</v>
+        <v>121</v>
       </c>
       <c r="D31" t="s">
-        <v>156</v>
+        <v>20</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>101</v>
+        <v>157</v>
       </c>
       <c r="B32" t="s">
-        <v>84</v>
+        <v>156</v>
       </c>
       <c r="C32" t="s">
-        <v>102</v>
+        <v>152</v>
       </c>
       <c r="D32" t="s">
-        <v>84</v>
+        <v>156</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
@@ -1532,7 +1523,7 @@
         <v>84</v>
       </c>
       <c r="C33" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D33" t="s">
         <v>84</v>
@@ -1546,7 +1537,7 @@
         <v>84</v>
       </c>
       <c r="C34" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D34" t="s">
         <v>84</v>
@@ -1554,44 +1545,44 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>127</v>
+        <v>101</v>
       </c>
       <c r="B35" t="s">
-        <v>125</v>
+        <v>84</v>
       </c>
       <c r="C35" t="s">
-        <v>126</v>
+        <v>104</v>
       </c>
       <c r="D35" t="s">
-        <v>125</v>
+        <v>84</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>67</v>
+        <v>127</v>
       </c>
       <c r="B36" t="s">
-        <v>66</v>
+        <v>125</v>
       </c>
       <c r="C36" t="s">
-        <v>67</v>
+        <v>126</v>
       </c>
       <c r="D36" t="s">
-        <v>68</v>
+        <v>125</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>164</v>
+        <v>67</v>
       </c>
       <c r="B37" t="s">
-        <v>125</v>
+        <v>66</v>
       </c>
       <c r="C37" t="s">
-        <v>165</v>
+        <v>67</v>
       </c>
       <c r="D37" t="s">
-        <v>125</v>
+        <v>68</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
@@ -1610,16 +1601,16 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>70</v>
+        <v>164</v>
       </c>
       <c r="B39" t="s">
-        <v>71</v>
+        <v>125</v>
       </c>
       <c r="C39" t="s">
-        <v>70</v>
+        <v>165</v>
       </c>
       <c r="D39" t="s">
-        <v>72</v>
+        <v>125</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
@@ -1633,7 +1624,7 @@
         <v>70</v>
       </c>
       <c r="D40" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
@@ -1647,21 +1638,21 @@
         <v>70</v>
       </c>
       <c r="D41" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>107</v>
+        <v>70</v>
       </c>
       <c r="B42" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C42" t="s">
-        <v>106</v>
+        <v>70</v>
       </c>
       <c r="D42" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
@@ -1672,7 +1663,7 @@
         <v>69</v>
       </c>
       <c r="C43" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D43" t="s">
         <v>69</v>
@@ -1686,7 +1677,7 @@
         <v>69</v>
       </c>
       <c r="C44" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="D44" t="s">
         <v>69</v>
@@ -1700,7 +1691,7 @@
         <v>69</v>
       </c>
       <c r="C45" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D45" t="s">
         <v>69</v>
@@ -1714,7 +1705,7 @@
         <v>69</v>
       </c>
       <c r="C46" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D46" t="s">
         <v>69</v>
@@ -1728,7 +1719,7 @@
         <v>69</v>
       </c>
       <c r="C47" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D47" t="s">
         <v>69</v>
@@ -1742,7 +1733,7 @@
         <v>69</v>
       </c>
       <c r="C48" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D48" t="s">
         <v>69</v>
@@ -1750,27 +1741,27 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>177</v>
+        <v>107</v>
       </c>
       <c r="B49" t="s">
-        <v>176</v>
+        <v>69</v>
       </c>
       <c r="C49" t="s">
-        <v>177</v>
+        <v>112</v>
       </c>
       <c r="D49" t="s">
-        <v>45</v>
+        <v>69</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B50" t="s">
-        <v>45</v>
+        <v>176</v>
       </c>
       <c r="C50" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D50" t="s">
         <v>45</v>
@@ -1778,16 +1769,16 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>139</v>
+        <v>178</v>
       </c>
       <c r="B51" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="C51" t="s">
-        <v>139</v>
+        <v>179</v>
       </c>
       <c r="D51" t="s">
-        <v>140</v>
+        <v>45</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
@@ -1801,7 +1792,7 @@
         <v>139</v>
       </c>
       <c r="D52" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
@@ -1815,7 +1806,7 @@
         <v>139</v>
       </c>
       <c r="D53" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
@@ -1829,21 +1820,21 @@
         <v>139</v>
       </c>
       <c r="D54" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>167</v>
+        <v>139</v>
       </c>
       <c r="B55" t="s">
-        <v>166</v>
+        <v>25</v>
       </c>
       <c r="C55" t="s">
-        <v>169</v>
+        <v>139</v>
       </c>
       <c r="D55" t="s">
-        <v>166</v>
+        <v>20</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
@@ -1854,7 +1845,7 @@
         <v>166</v>
       </c>
       <c r="C56" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D56" t="s">
         <v>166</v>
@@ -1862,58 +1853,58 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>131</v>
+        <v>167</v>
       </c>
       <c r="B57" t="s">
-        <v>132</v>
+        <v>166</v>
       </c>
       <c r="C57" t="s">
-        <v>133</v>
+        <v>170</v>
       </c>
       <c r="D57" t="s">
-        <v>132</v>
+        <v>166</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>5</v>
+        <v>131</v>
       </c>
       <c r="B58" t="s">
-        <v>6</v>
+        <v>132</v>
       </c>
       <c r="C58" t="s">
-        <v>5</v>
+        <v>133</v>
       </c>
       <c r="D58" t="s">
-        <v>7</v>
+        <v>132</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>197</v>
+        <v>5</v>
       </c>
       <c r="B59" t="s">
-        <v>196</v>
+        <v>6</v>
       </c>
       <c r="C59" t="s">
-        <v>109</v>
+        <v>5</v>
       </c>
       <c r="D59" t="s">
-        <v>196</v>
+        <v>7</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>78</v>
+        <v>196</v>
       </c>
       <c r="B60" t="s">
-        <v>79</v>
+        <v>195</v>
       </c>
       <c r="C60" t="s">
-        <v>78</v>
+        <v>109</v>
       </c>
       <c r="D60" t="s">
-        <v>80</v>
+        <v>195</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
@@ -1927,21 +1918,21 @@
         <v>78</v>
       </c>
       <c r="D61" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="B62" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="C62" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="D62" t="s">
-        <v>60</v>
+        <v>81</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
@@ -1955,21 +1946,21 @@
         <v>62</v>
       </c>
       <c r="D63" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="B64" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="C64" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="D64" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
@@ -1983,7 +1974,7 @@
         <v>21</v>
       </c>
       <c r="D65" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
@@ -1994,10 +1985,10 @@
         <v>20</v>
       </c>
       <c r="C66" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="D66" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
@@ -2008,7 +1999,7 @@
         <v>20</v>
       </c>
       <c r="C67" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="D67" t="s">
         <v>22</v>
@@ -2025,7 +2016,7 @@
         <v>24</v>
       </c>
       <c r="D68" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.2">
@@ -2039,7 +2030,7 @@
         <v>24</v>
       </c>
       <c r="D69" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
@@ -2053,35 +2044,35 @@
         <v>24</v>
       </c>
       <c r="D70" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>144</v>
+        <v>21</v>
       </c>
       <c r="B71" t="s">
-        <v>143</v>
+        <v>20</v>
       </c>
       <c r="C71" t="s">
-        <v>145</v>
+        <v>24</v>
       </c>
       <c r="D71" t="s">
-        <v>143</v>
+        <v>40</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>63</v>
+        <v>144</v>
       </c>
       <c r="B72" t="s">
-        <v>64</v>
+        <v>143</v>
       </c>
       <c r="C72" t="s">
-        <v>65</v>
+        <v>145</v>
       </c>
       <c r="D72" t="s">
-        <v>64</v>
+        <v>143</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
@@ -2100,58 +2091,58 @@
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>175</v>
+        <v>63</v>
       </c>
       <c r="B74" t="s">
-        <v>154</v>
+        <v>64</v>
       </c>
       <c r="C74" t="s">
-        <v>175</v>
+        <v>65</v>
       </c>
       <c r="D74" t="s">
-        <v>153</v>
+        <v>64</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>57</v>
+        <v>175</v>
       </c>
       <c r="B75" t="s">
-        <v>52</v>
+        <v>154</v>
       </c>
       <c r="C75" t="s">
-        <v>57</v>
+        <v>175</v>
       </c>
       <c r="D75" t="s">
-        <v>58</v>
+        <v>153</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>185</v>
+        <v>57</v>
       </c>
       <c r="B76" t="s">
-        <v>142</v>
+        <v>52</v>
       </c>
       <c r="C76" t="s">
-        <v>185</v>
+        <v>57</v>
       </c>
       <c r="D76" t="s">
-        <v>20</v>
+        <v>58</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>59</v>
+        <v>185</v>
       </c>
       <c r="B77" t="s">
-        <v>52</v>
+        <v>142</v>
       </c>
       <c r="C77" t="s">
-        <v>59</v>
+        <v>185</v>
       </c>
       <c r="D77" t="s">
-        <v>58</v>
+        <v>20</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.2">
@@ -2165,49 +2156,49 @@
         <v>59</v>
       </c>
       <c r="D78" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>173</v>
+        <v>59</v>
       </c>
       <c r="B79" t="s">
-        <v>174</v>
+        <v>52</v>
       </c>
       <c r="C79" t="s">
-        <v>172</v>
+        <v>59</v>
       </c>
       <c r="D79" t="s">
-        <v>174</v>
+        <v>60</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>39</v>
+        <v>173</v>
       </c>
       <c r="B80" t="s">
-        <v>20</v>
+        <v>174</v>
       </c>
       <c r="C80" t="s">
-        <v>39</v>
+        <v>172</v>
       </c>
       <c r="D80" t="s">
-        <v>22</v>
+        <v>174</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="B81" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="C81" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="D81" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.2">
@@ -2221,7 +2212,7 @@
         <v>12</v>
       </c>
       <c r="D82" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.2">
@@ -2232,7 +2223,7 @@
         <v>11</v>
       </c>
       <c r="C83" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D83" t="s">
         <v>14</v>
@@ -2240,16 +2231,16 @@
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>187</v>
+        <v>12</v>
       </c>
       <c r="B84" t="s">
-        <v>74</v>
+        <v>11</v>
       </c>
       <c r="C84" t="s">
-        <v>137</v>
+        <v>15</v>
       </c>
       <c r="D84" t="s">
-        <v>138</v>
+        <v>14</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.2">
@@ -2263,7 +2254,7 @@
         <v>137</v>
       </c>
       <c r="D85" t="s">
-        <v>74</v>
+        <v>138</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.2">
@@ -2274,10 +2265,10 @@
         <v>74</v>
       </c>
       <c r="C86" t="s">
-        <v>150</v>
+        <v>137</v>
       </c>
       <c r="D86" t="s">
-        <v>138</v>
+        <v>74</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.2">
@@ -2288,10 +2279,10 @@
         <v>74</v>
       </c>
       <c r="C87" t="s">
-        <v>137</v>
+        <v>150</v>
       </c>
       <c r="D87" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.2">
@@ -2302,38 +2293,38 @@
         <v>74</v>
       </c>
       <c r="C88" t="s">
-        <v>187</v>
+        <v>137</v>
       </c>
       <c r="D88" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>36</v>
+        <v>187</v>
       </c>
       <c r="B89" t="s">
-        <v>31</v>
+        <v>74</v>
       </c>
       <c r="C89" t="s">
-        <v>37</v>
+        <v>187</v>
       </c>
       <c r="D89" t="s">
-        <v>31</v>
+        <v>138</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="B90" t="s">
-        <v>52</v>
+        <v>31</v>
       </c>
       <c r="C90" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="D90" t="s">
-        <v>52</v>
+        <v>31</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.2">
@@ -2344,7 +2335,7 @@
         <v>52</v>
       </c>
       <c r="C91" t="s">
-        <v>188</v>
+        <v>53</v>
       </c>
       <c r="D91" t="s">
         <v>52</v>
@@ -2352,30 +2343,30 @@
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B92" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C92" t="s">
-        <v>54</v>
+        <v>188</v>
       </c>
       <c r="D92" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>3</v>
+        <v>54</v>
       </c>
       <c r="B93" t="s">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="C93" t="s">
-        <v>1</v>
+        <v>54</v>
       </c>
       <c r="D93" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.2">
@@ -2389,7 +2380,7 @@
         <v>1</v>
       </c>
       <c r="D94" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.2">
@@ -2400,10 +2391,10 @@
         <v>0</v>
       </c>
       <c r="C95" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D95" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.2">
@@ -2417,21 +2408,21 @@
         <v>3</v>
       </c>
       <c r="D96" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>89</v>
+        <v>3</v>
       </c>
       <c r="B97" t="s">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="C97" t="s">
-        <v>89</v>
+        <v>3</v>
       </c>
       <c r="D97" t="s">
-        <v>88</v>
+        <v>4</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.2">
@@ -2445,46 +2436,46 @@
         <v>89</v>
       </c>
       <c r="D98" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>8</v>
+        <v>89</v>
       </c>
       <c r="B99" t="s">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="C99" t="s">
-        <v>9</v>
+        <v>89</v>
       </c>
       <c r="D99" t="s">
-        <v>10</v>
+        <v>91</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>44</v>
+        <v>8</v>
       </c>
       <c r="B100" t="s">
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="C100" t="s">
-        <v>44</v>
+        <v>9</v>
       </c>
       <c r="D100" t="s">
-        <v>45</v>
+        <v>10</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>181</v>
+        <v>44</v>
       </c>
       <c r="B101" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C101" t="s">
-        <v>180</v>
+        <v>44</v>
       </c>
       <c r="D101" t="s">
         <v>45</v>
@@ -2498,7 +2489,7 @@
         <v>45</v>
       </c>
       <c r="C102" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D102" t="s">
         <v>45</v>
@@ -2512,7 +2503,7 @@
         <v>45</v>
       </c>
       <c r="C103" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D103" t="s">
         <v>45</v>
@@ -2526,10 +2517,10 @@
         <v>45</v>
       </c>
       <c r="C104" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="D104" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.2">
@@ -2540,10 +2531,10 @@
         <v>45</v>
       </c>
       <c r="C105" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="D105" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.2">
@@ -2554,7 +2545,7 @@
         <v>45</v>
       </c>
       <c r="C106" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D106" t="s">
         <v>45</v>
@@ -2562,212 +2553,212 @@
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>159</v>
+        <v>181</v>
       </c>
       <c r="B107" t="s">
-        <v>151</v>
+        <v>45</v>
       </c>
       <c r="C107" t="s">
-        <v>159</v>
+        <v>184</v>
       </c>
       <c r="D107" t="s">
-        <v>154</v>
+        <v>45</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>159</v>
+        <v>191</v>
       </c>
       <c r="B108" t="s">
-        <v>151</v>
+        <v>193</v>
       </c>
       <c r="C108" t="s">
-        <v>159</v>
+        <v>192</v>
       </c>
       <c r="D108" t="s">
-        <v>153</v>
+        <v>193</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B109" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="C109" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D109" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B110" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
       <c r="C110" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D110" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
-        <v>92</v>
+        <v>161</v>
       </c>
       <c r="B111" t="s">
-        <v>79</v>
+        <v>160</v>
       </c>
       <c r="C111" t="s">
-        <v>92</v>
+        <v>161</v>
       </c>
       <c r="D111" t="s">
-        <v>81</v>
+        <v>162</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>92</v>
+        <v>161</v>
       </c>
       <c r="B112" t="s">
-        <v>79</v>
+        <v>160</v>
       </c>
       <c r="C112" t="s">
-        <v>92</v>
+        <v>161</v>
       </c>
       <c r="D112" t="s">
-        <v>80</v>
+        <v>163</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
-        <v>26</v>
+        <v>92</v>
       </c>
       <c r="B113" t="s">
-        <v>25</v>
+        <v>79</v>
       </c>
       <c r="C113" t="s">
-        <v>20</v>
+        <v>92</v>
       </c>
       <c r="D113" t="s">
-        <v>26</v>
+        <v>81</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
-        <v>190</v>
+        <v>92</v>
       </c>
       <c r="B114" t="s">
-        <v>141</v>
+        <v>79</v>
       </c>
       <c r="C114" t="s">
-        <v>190</v>
+        <v>92</v>
       </c>
       <c r="D114" t="s">
-        <v>40</v>
+        <v>80</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B115" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="C115" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D115" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
-        <v>209</v>
+        <v>190</v>
       </c>
       <c r="B116" t="s">
-        <v>194</v>
+        <v>141</v>
       </c>
       <c r="C116" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D116" t="s">
-        <v>194</v>
+        <v>40</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
-        <v>209</v>
+        <v>24</v>
       </c>
       <c r="B117" t="s">
-        <v>194</v>
+        <v>42</v>
       </c>
       <c r="C117" t="s">
-        <v>193</v>
+        <v>24</v>
       </c>
       <c r="D117" t="s">
-        <v>194</v>
+        <v>41</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B118" t="s">
-        <v>194</v>
+        <v>45</v>
       </c>
       <c r="C118" t="s">
-        <v>192</v>
+        <v>207</v>
       </c>
       <c r="D118" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
-        <v>209</v>
+        <v>96</v>
       </c>
       <c r="B119" t="s">
-        <v>194</v>
+        <v>95</v>
       </c>
       <c r="C119" t="s">
-        <v>210</v>
+        <v>97</v>
       </c>
       <c r="D119" t="s">
-        <v>194</v>
+        <v>95</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
-        <v>208</v>
+        <v>46</v>
       </c>
       <c r="B120" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C120" t="s">
-        <v>208</v>
+        <v>48</v>
       </c>
       <c r="D120" t="s">
-        <v>207</v>
+        <v>47</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
-        <v>96</v>
+        <v>46</v>
       </c>
       <c r="B121" t="s">
-        <v>95</v>
+        <v>47</v>
       </c>
       <c r="C121" t="s">
-        <v>97</v>
+        <v>49</v>
       </c>
       <c r="D121" t="s">
-        <v>95</v>
+        <v>47</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.2">
@@ -2778,127 +2769,85 @@
         <v>47</v>
       </c>
       <c r="C122" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D122" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
-        <v>46</v>
+        <v>198</v>
       </c>
       <c r="B123" t="s">
-        <v>47</v>
+        <v>197</v>
       </c>
       <c r="C123" t="s">
-        <v>49</v>
-      </c>
-      <c r="D123" t="s">
-        <v>47</v>
+        <v>199</v>
+      </c>
+      <c r="D123" s="3" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
-        <v>46</v>
+        <v>198</v>
       </c>
       <c r="B124" t="s">
-        <v>47</v>
+        <v>197</v>
       </c>
       <c r="C124" t="s">
-        <v>49</v>
-      </c>
-      <c r="D124" t="s">
-        <v>50</v>
+        <v>200</v>
+      </c>
+      <c r="D124" s="3" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="B125" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="C125" t="s">
-        <v>200</v>
-      </c>
-      <c r="D125" s="3" t="s">
-        <v>198</v>
+        <v>204</v>
+      </c>
+      <c r="D125" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
-        <v>199</v>
+        <v>82</v>
       </c>
       <c r="B126" t="s">
-        <v>198</v>
+        <v>83</v>
       </c>
       <c r="C126" t="s">
-        <v>201</v>
-      </c>
-      <c r="D126" s="3" t="s">
-        <v>198</v>
+        <v>82</v>
+      </c>
+      <c r="D126" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
-        <v>205</v>
+        <v>82</v>
       </c>
       <c r="B127" t="s">
-        <v>206</v>
+        <v>83</v>
       </c>
       <c r="C127" t="s">
-        <v>205</v>
+        <v>82</v>
       </c>
       <c r="D127" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A128" t="s">
-        <v>82</v>
-      </c>
-      <c r="B128" t="s">
-        <v>83</v>
-      </c>
-      <c r="C128" t="s">
-        <v>82</v>
-      </c>
-      <c r="D128" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A129" t="s">
-        <v>82</v>
-      </c>
-      <c r="B129" t="s">
-        <v>83</v>
-      </c>
-      <c r="C129" t="s">
-        <v>82</v>
-      </c>
-      <c r="D129" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A130" t="s">
-        <v>109</v>
-      </c>
-      <c r="B130" t="s">
-        <v>74</v>
-      </c>
-      <c r="C130" t="s">
-        <v>109</v>
-      </c>
-      <c r="D130" t="s">
-        <v>138</v>
-      </c>
-    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D129">
-    <sortCondition ref="A2:A129"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D127">
+    <sortCondition ref="A2:A127"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
minor validation updates while looking through final output
</commit_message>
<xml_diff>
--- a/src/inputs/canonical_nodes.xlsx
+++ b/src/inputs/canonical_nodes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ben/Documents/bruegel/data_new/WORKING/INDUSTRY/tuone_v6/src/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99275586-62D6-3048-A7B3-0D1B93B3CB46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BED330E3-13D9-834A-8EBE-531F51C7AA42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="800" windowWidth="29400" windowHeight="16940" xr2:uid="{EBC50A8D-91C7-594D-A950-AF99F2B3F4AF}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16940" xr2:uid="{EBC50A8D-91C7-594D-A950-AF99F2B3F4AF}"/>
   </bookViews>
   <sheets>
     <sheet name="merge" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="211">
   <si>
     <t>Pylon LifeEU</t>
   </si>
@@ -661,6 +661,15 @@
   </si>
   <si>
     <t>Västerås</t>
+  </si>
+  <si>
+    <t>Rainbach, Mühlkreis</t>
+  </si>
+  <si>
+    <t>Kreisel Electric</t>
+  </si>
+  <si>
+    <t>Rainbach</t>
   </si>
 </sst>
 </file>
@@ -1056,7 +1065,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DF9B3CA-7DC7-BB45-882F-C1DDB5BD93A3}">
-  <dimension ref="A1:E127"/>
+  <dimension ref="A1:E128"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.5" bestFit="1" customWidth="1"/>
@@ -2843,6 +2852,20 @@
       </c>
       <c r="D127" t="s">
         <v>84</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A128" t="s">
+        <v>210</v>
+      </c>
+      <c r="B128" t="s">
+        <v>209</v>
+      </c>
+      <c r="C128" t="s">
+        <v>208</v>
+      </c>
+      <c r="D128" t="s">
+        <v>209</v>
       </c>
     </row>
   </sheetData>

</xml_diff>